<commit_message>
Refined Gasket Header+ Waste Material
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -421,11 +421,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="76" customWidth="1" min="5" max="5"/>
@@ -459,7 +459,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="25">
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>MANUAL PART-NUMBERED ITEMS</t>
+          <t>GLASS</t>
         </is>
       </c>
     </row>
@@ -1008,27 +1008,27 @@
     <row r="27">
       <c r="E27" t="inlineStr">
         <is>
-          <t>Gasket</t>
+          <t>Glass Area</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>E2-0052</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0.6666666666666666 ft</t>
+          <t>0.0625 sqft</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>405</v>
+        <v>0.65625</v>
       </c>
     </row>
     <row r="28">
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>GLASS</t>
+          <t>FABRICATION</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
     <row r="30">
       <c r="E30" t="inlineStr">
         <is>
-          <t>Glass Area</t>
+          <t>Joints Fabrication Labor</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1067,17 +1067,17 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0.0625 sqft</t>
+          <t>4 joints</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>0.65625</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31">
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>FABRICATION</t>
+          <t>GLAZING GASKET</t>
         </is>
       </c>
     </row>
@@ -1106,21 +1106,21 @@
     <row r="33">
       <c r="E33" t="inlineStr">
         <is>
-          <t>Joints Fabrication Labor</t>
+          <t>Gasket</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>E2-0052</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>4 joints</t>
+          <t>0.6666666666666666 ft</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>60</v>
+        <v>405</v>
       </c>
     </row>
     <row r="34">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E37" s="1" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0.16666666666666666 ft</t>
+          <t>16.0 ft</t>
         </is>
       </c>
       <c r="H38" s="2" t="n">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1233,11 +1233,11 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0.08333333333333333 ft</t>
+          <t>12.0 ft</t>
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>0</v>
+        <v>502.8</v>
       </c>
     </row>
     <row r="40">
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1261,11 +1261,11 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>0.0 ft</t>
+          <t>24.0 ft</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="41">
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>144</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1289,11 +1289,11 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>0.0 ft</t>
+          <t>24.0 ft</t>
         </is>
       </c>
       <c r="H41" s="2" t="n">
-        <v>0</v>
+        <v>596.4</v>
       </c>
     </row>
     <row r="42">
@@ -1303,7 +1303,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>96</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>0.08333333333333333 ft</t>
+          <t>12.0 ft</t>
         </is>
       </c>
       <c r="H42" s="2" t="n">
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.006944444444444444</v>
+        <v>96</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>0.08333333333333333 ft</t>
+          <t>12.0 ft</t>
         </is>
       </c>
       <c r="H43" s="2" t="n">
@@ -1359,7 +1359,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.006944444444444444</v>
+        <v>96</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>0.08333333333333333 ft</t>
+          <t>12.0 ft</t>
         </is>
       </c>
       <c r="H44" s="2" t="n">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.3333333333333333</v>
+        <v>40</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1401,11 +1401,11 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>0.08333333333333333 ft</t>
+          <t>24.0 ft</t>
         </is>
       </c>
       <c r="H45" s="2" t="n">
-        <v>0</v>
+        <v>102.06</v>
       </c>
     </row>
     <row r="46">
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.3333333333333333</v>
+        <v>40</v>
       </c>
     </row>
     <row r="47">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>3' X 8'</t>
         </is>
       </c>
       <c r="E47" s="1" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2 pcs</t>
+          <t>8 pcs</t>
         </is>
       </c>
       <c r="H50" s="2" t="n">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>8 pcs</t>
+          <t>56 pcs</t>
         </is>
       </c>
       <c r="H51" s="2" t="n">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>3 pcs</t>
+          <t>12 pcs</t>
         </is>
       </c>
       <c r="H52" s="2" t="n">
@@ -1570,11 +1570,11 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2 pcs</t>
+          <t>8 pcs</t>
         </is>
       </c>
       <c r="H54" s="2" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="55">
@@ -1590,11 +1590,11 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>0 pcs</t>
+          <t>6 pcs</t>
         </is>
       </c>
       <c r="H55" s="2" t="n">
-        <v>0</v>
+        <v>76.95</v>
       </c>
     </row>
     <row r="56">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2 pcs</t>
+          <t>8 pcs</t>
         </is>
       </c>
       <c r="H56" s="2" t="n">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2 pcs</t>
+          <t>4 pcs</t>
         </is>
       </c>
       <c r="H57" s="2" t="n">
@@ -1650,11 +1650,11 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>0 pcs</t>
+          <t>6 pcs</t>
         </is>
       </c>
       <c r="H58" s="2" t="n">
-        <v>0</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="59">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2 pcs</t>
+          <t>8 pcs</t>
         </is>
       </c>
       <c r="H59" s="2" t="n">
@@ -1680,7 +1680,7 @@
     <row r="60">
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>MANUAL PART-NUMBERED ITEMS</t>
+          <t>GLASS</t>
         </is>
       </c>
     </row>
@@ -1709,27 +1709,27 @@
     <row r="62">
       <c r="E62" t="inlineStr">
         <is>
-          <t>Gasket</t>
+          <t>Glass Area</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>E2-0052</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>0.6666666666666666 ft</t>
+          <t>59.75 sqft</t>
         </is>
       </c>
       <c r="H62" s="2" t="n">
-        <v>0</v>
+        <v>627.375</v>
       </c>
     </row>
     <row r="63">
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>GLASS</t>
+          <t>DOOR</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1758,7 @@
     <row r="65">
       <c r="E65" t="inlineStr">
         <is>
-          <t>Glass Area</t>
+          <t>Door</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -1768,11 +1768,11 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>0.0625 sqft</t>
+          <t>24.0 sqft</t>
         </is>
       </c>
       <c r="H65" s="2" t="n">
-        <v>0.65625</v>
+        <v>240</v>
       </c>
     </row>
     <row r="66">
@@ -1817,282 +1817,247 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>4 joints</t>
+          <t>24 joints</t>
         </is>
       </c>
       <c r="H68" s="2" t="n">
-        <v>60</v>
+        <v>360</v>
       </c>
     </row>
     <row r="69">
-      <c r="H69" s="1" t="inlineStr">
+      <c r="E69" s="1" t="inlineStr">
+        <is>
+          <t>GLAZING GASKET</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="E70" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F70" s="1" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="H70" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Gasket</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>E2-0052</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>224.0 ft</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="H72" s="1" t="inlineStr">
         <is>
           <t>SYSTEM TOTAL</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="H70" s="2" t="n">
-        <v>69.65625</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="H71" s="1" t="inlineStr">
+    <row r="73">
+      <c r="H73" s="2" t="n">
+        <v>2778.285</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="H74" s="1" t="inlineStr">
         <is>
           <t>RUNNING GRAND TOTAL</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="H72" s="2" t="n">
-        <v>2899.9125</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="1" t="inlineStr">
+    <row r="75">
+      <c r="H75" s="2" t="n">
+        <v>5608.54125</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr">
         <is>
           <t>Part Number / Description</t>
         </is>
       </c>
-      <c r="B73" s="1" t="inlineStr">
+      <c r="B76" s="1" t="inlineStr">
         <is>
           <t>Total Quantity</t>
         </is>
       </c>
-      <c r="C73" s="1" t="inlineStr">
+      <c r="C76" s="1" t="inlineStr">
         <is>
           <t>Total Price</t>
         </is>
       </c>
-      <c r="D73" s="1" t="inlineStr">
+      <c r="D76" s="1" t="inlineStr">
         <is>
           <t>Reusable Material Quantity</t>
         </is>
       </c>
-      <c r="E73" s="1" t="inlineStr">
+      <c r="E76" s="1" t="inlineStr">
         <is>
           <t>Reusable % of Total</t>
         </is>
       </c>
-      <c r="F73" s="1" t="inlineStr">
+      <c r="F76" s="1" t="inlineStr">
         <is>
           <t>Reusable Material Cost</t>
         </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>E1-0199</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>4.0 pcs</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="n">
-        <v>64.8</v>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>16.00 pcs</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="inlineStr">
-        <is>
-          <t>400.00%</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="n">
-        <v>51.84</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>E2-0047</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>4.0 pcs</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>46.00 pcs</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>1150.00%</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="n">
-        <v>109.48</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>PC-1220</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>16.0 pcs</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="n">
-        <v>18.3</v>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>84.00 pcs</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr">
-        <is>
-          <t>525.00%</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="n">
-        <v>15.372</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PM-1006-SS</t>
+          <t>E1-0199</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>6.0 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
-        <v>46.65</v>
+        <v>64.8</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>94.00 pcs</t>
+          <t>16.00 pcs</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>1566.67%</t>
+          <t>400.00%</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>43.851</v>
+        <v>51.84</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>UA-1212</t>
+          <t>E2-0047</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>8.0 pcs</t>
+          <t>10.00 pcs</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
-        <v>48.6</v>
+        <v>119</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>92.00 pcs</t>
+          <t>40.00 pcs</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>1150.00%</t>
+          <t>400.00%</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>44.712</v>
+        <v>95.19999999999999</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>E1-2530</t>
+          <t>PC-1220</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>4.0 pcs</t>
+          <t>64.00 pcs</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
-        <v>18</v>
+        <v>18.3</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>36.00 pcs</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>56.25%</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
-        <v>0</v>
+        <v>6.588</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>E2-0166</t>
+          <t>PM-1006-SS</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>0.0 pcs</t>
+          <t>15.00 pcs</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
-        <v>0</v>
+        <v>46.65</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>85.00 pcs</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>566.67%</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>0</v>
+        <v>39.6525</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>E2-0177</t>
+          <t>UA-1212</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>4.0 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
-        <v>76.95</v>
+        <v>48.6</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>46.00 pcs</t>
+          <t>92.00 pcs</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
@@ -2101,342 +2066,454 @@
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>70.79400000000001</v>
+        <v>44.712</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>E2-0545</t>
+          <t>E1-2530</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>4.0 pcs</t>
+          <t>10.00 pcs</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
-        <v>147</v>
+        <v>45</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>46.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>1150.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>135.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>E2-0154</t>
+          <t>E2-0166</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>0.0 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
-        <v>0</v>
+        <v>76.95</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>733.33%</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>0</v>
+        <v>67.71600000000001</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>E2-0611</t>
+          <t>E2-0177</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>4.0 pcs</t>
+          <t>10.00 pcs</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
-        <v>95.25</v>
+        <v>76.95</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>46.00 pcs</t>
+          <t>40.00 pcs</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>1150.00%</t>
+          <t>400.00%</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>87.63</v>
+        <v>61.56</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>BE9-2513</t>
+          <t>E2-0545</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>0.49999999999999994 ft</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
-        <v>419</v>
+        <v>147</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>23.50 ft</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>4700.00%</t>
+          <t>733.33%</t>
         </is>
       </c>
       <c r="F85" s="2" t="n">
-        <v>410.2708333333333</v>
+        <v>129.36</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>E9-2512</t>
+          <t>E2-0154</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>0.0 ft</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
-        <v>0</v>
+        <v>56.7</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>733.33%</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>0</v>
+        <v>49.89600000000001</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>BE9-2511</t>
+          <t>E2-0611</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>0.0 ft</t>
+          <t>10.00 pcs</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
-        <v>0</v>
+        <v>95.25</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>40.00 pcs</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>400.00%</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>0</v>
+        <v>76.2</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>BE9-2515</t>
+          <t>BE9-2513</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>0.16666666666666666 ft</t>
+          <t>28.25 ft</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
-        <v>527</v>
+        <v>838</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>23.83 ft</t>
+          <t>19.75 ft</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>14300.00%</t>
+          <t>69.91%</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>523.3402777777778</v>
+        <v>344.8020833333333</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>BE9-2514</t>
+          <t>E9-2512</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>0.16666666666666666 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
-        <v>444</v>
+        <v>150</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>23.83 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>14300.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>440.9166666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BE9-2578</t>
+          <t>BE9-2511</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>0.16666666666666666 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
-        <v>264</v>
+        <v>497</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>23.83 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>14300.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>262.1666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>E9-2519</t>
+          <t>BE9-2515</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>0.16666666666666666 ft</t>
+          <t>12.08 ft</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
-        <v>85.05</v>
+        <v>527</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>23.83 ft</t>
+          <t>11.92 ft</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>14300.00%</t>
+          <t>98.62%</t>
         </is>
       </c>
       <c r="F91" s="2" t="n">
-        <v>84.45937500000001</v>
+        <v>261.6701388888889</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Glass Area</t>
+          <t>BE9-2514</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>0.125 sqft</t>
+          <t>12.08 ft</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
-        <v>1.3125</v>
-      </c>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" s="3" t="inlineStr"/>
-      <c r="F92" s="2" t="inlineStr"/>
+        <v>444</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>11.92 ft</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>98.62%</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>220.4583333333333</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Joints Fabrication Labor</t>
+          <t>BE9-2578</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>8.0 joints</t>
+          <t>12.08 ft</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
-        <v>120</v>
-      </c>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" s="3" t="inlineStr"/>
-      <c r="F93" s="2" t="inlineStr"/>
+        <v>264</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>11.92 ft</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>98.62%</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="n">
+        <v>131.0833333333333</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
+          <t>E9-2519</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>24.08 ft</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="n">
+        <v>170.1</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>23.92 ft</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>99.31%</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="n">
+        <v>84.7546875</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Glass Area</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>59.81 sqft</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="n">
+        <v>628.03125</v>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" s="3" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Joints Fabrication Labor</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>28.00 joints</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" s="3" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
           <t>Gasket (E2-0052)</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>1.3333333333333333 ft</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="n">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>224.67 ft</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="n">
         <v>405</v>
       </c>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" s="3" t="inlineStr"/>
-      <c r="F94" s="2" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>275.33 ft</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>122.55%</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>223.02</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Door</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>24.00 sqft</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" s="3" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Just needs to add door to system
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -51,10 +51,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,15 +421,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="2" customWidth="1" min="3" max="3"/>
-    <col width="2" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="76" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
@@ -444,6 +445,11 @@
           <t>YES 45TU FRONT SET(OG)</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PROFILES</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -456,6 +462,26 @@
           <t>Clear</t>
         </is>
       </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -468,6 +494,24 @@
           <t>1</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sill/Jamb Screw Spline Assembly</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>BE9-2513</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>16.00 ft</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>419</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -478,6 +522,24 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sill/Jamb Screw Spline Assembly</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>BE9-2513</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>12.00 ft</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>419</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -488,6 +550,24 @@
       <c r="B5" t="n">
         <v>4</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Flush Filler</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>E9-2512</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>24.00 ft</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -498,6 +578,24 @@
       <c r="B6" t="n">
         <v>2</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Two Piece Mullion Screw Spline Assembly</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BE9-2511</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>24.00 ft</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>497</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -508,6 +606,24 @@
       <c r="B7" t="n">
         <v>144</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Horizontal Screw Spline Assembly</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BE9-2515</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>12.00 ft</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>527</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -518,6 +634,24 @@
       <c r="B8" t="n">
         <v>96</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BE9-2514</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>12.00 ft</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>444</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -528,6 +662,24 @@
       <c r="B9" t="n">
         <v>96</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Thermal Sill Flashing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>BE9-2578</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>12.00 ft</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>264</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -538,6 +690,24 @@
       <c r="B10" t="n">
         <v>96</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Glass Stop (Use with BE9-2514, BE9-2515, BE9-2517)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>E9-2519</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>24.00 ft</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>85.05</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -558,157 +728,183 @@
       <c r="B12" t="n">
         <v>40</v>
       </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>ACCESSORIES</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>Doors</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1x 3' X 8' Narrow with Continuous Hinges, Concealed Closer</t>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>ACCESSORIES</t>
-        </is>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>End Dam For Sill Flashing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>E1-0199</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2.00 pcs</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>64.8</v>
       </c>
     </row>
     <row r="15">
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G15" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H15" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Water Deflector</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>E2-0047</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="16">
       <c r="E16" t="inlineStr">
         <is>
-          <t>End Dam For Sill Flashing</t>
+          <t>#12 x 1-1/4” PHSMS Type AB, Zinc Plated Steel, For Screw Spline Attachment</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>E1-0199</t>
+          <t>PC-1220</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>56.00 pcs</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>64.8</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="17">
       <c r="E17" t="inlineStr">
         <is>
-          <t>Water Deflector</t>
+          <t>#10-24 x 3/8” PHMS, Stainless Steel, For Attachment of Sill to Sill Flashing</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>E2-0047</t>
+          <t>PM-1006-SS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>12.00 pcs</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>119</v>
+        <v>46.65</v>
       </c>
     </row>
     <row r="18">
       <c r="E18" t="inlineStr">
         <is>
-          <t>#12 x 1-1/4” PHSMS Type AB, Zinc Plated Steel, For Screw Spline Attachment</t>
+          <t>#12 x 3/4” UFHSMS Type A, Zinc Plated Steel For End Dam Attachment</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PC-1220</t>
+          <t>UA-1212</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>56.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>18.3</v>
+        <v>48.6</v>
       </c>
     </row>
     <row r="19">
       <c r="E19" t="inlineStr">
         <is>
-          <t>#10-24 x 3/8” PHMS, Stainless Steel, For Attachment of Sill to Sill Flashing</t>
+          <t>Setting Block Chair Use with E2-0177 Setting Block at Sill</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PM-1006-SS</t>
+          <t>E1-2530</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46.65</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20">
       <c r="E20" t="inlineStr">
         <is>
-          <t>#12 x 3/4” UFHSMS Type A, Zinc Plated Steel For End Dam Attachment</t>
+          <t>Side Block For Intermediate Vertical Shallow Pocket</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>UA-1212</t>
+          <t>E2-0166</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>48.6</v>
+        <v>76.95</v>
       </c>
     </row>
     <row r="21">
       <c r="E21" t="inlineStr">
         <is>
-          <t>Setting Block Chair Use with E2-0177 Setting Block at Sill</t>
+          <t>Setting Block For Sill</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>E1-2530</t>
+          <t>E2-0177</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -717,516 +913,876 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>36</v>
+        <v>76.95</v>
       </c>
     </row>
     <row r="22">
       <c r="E22" t="inlineStr">
         <is>
-          <t>Side Block For Intermediate Vertical Shallow Pocket</t>
+          <t>1-1/8” “W” Side Block For Jamb</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>E2-0166</t>
+          <t>E2-0545</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>6.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>76.95</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23">
       <c r="E23" t="inlineStr">
         <is>
-          <t>Setting Block For Sill</t>
+          <t>1/2” “W” Side Block For Intermediate Vertical Deep Pocket</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>E2-0177</t>
+          <t>E2-0154</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>76.95</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="24">
       <c r="E24" t="inlineStr">
         <is>
-          <t>1-1/8” “W” Side Block For Jamb</t>
+          <t>Setting Block For Intermediate Horizontal</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>E2-0545</t>
+          <t>E2-0611</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>147</v>
+        <v>95.25</v>
       </c>
     </row>
     <row r="25">
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>1/2” “W” Side Block For Intermediate Vertical Deep Pocket</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>E2-0154</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>6.00 pcs</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>56.7</v>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>GLASS</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Setting Block For Intermediate Horizontal</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>E2-0611</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>8.00 pcs</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>95.25</v>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
       </c>
     </row>
     <row r="27">
-      <c r="E27" s="1" t="inlineStr">
-        <is>
-          <t>DOORS</t>
-        </is>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Glass Area</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>83.75 sqft</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>879.375</v>
       </c>
     </row>
     <row r="28">
       <c r="E28" s="1" t="inlineStr">
         <is>
+          <t>FABRICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="E29" s="1" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>Part Number</t>
         </is>
       </c>
-      <c r="G28" s="1" t="inlineStr">
+      <c r="G29" s="1" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="H28" s="1" t="inlineStr">
+      <c r="H29" s="1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Door (3' X 8') - Stile: Narrow</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+    <row r="30">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Joints Fabrication Labor</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="n">
-        <v>1488</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="E30" s="1" t="inlineStr">
-        <is>
-          <t>PROFILES</t>
-        </is>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>24.00 joints</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>360</v>
       </c>
     </row>
     <row r="31">
       <c r="E31" s="1" t="inlineStr">
         <is>
+          <t>GLAZING GASKET</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" s="1" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>Part Number</t>
         </is>
       </c>
-      <c r="G31" s="1" t="inlineStr">
+      <c r="G32" s="1" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="H31" s="1" t="inlineStr">
+      <c r="H32" s="1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Sill/Jamb Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>BE9-2513</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>16.00 ft</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="n">
-        <v>419</v>
       </c>
     </row>
     <row r="33">
       <c r="E33" t="inlineStr">
         <is>
-          <t>Sill/Jamb Screw Spline Assembly</t>
+          <t>Gasket</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>BE9-2513</t>
+          <t>E2-0052</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
+          <t>224.00 ft</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="H34" s="1" t="inlineStr">
+        <is>
+          <t>SYSTEM TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="H35" s="2" t="n">
+        <v>5235.625</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="H36" s="1" t="inlineStr">
+        <is>
+          <t>RUNNING GRAND TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="H37" s="2" t="n">
+        <v>5235.625</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>Part Number / Description</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>Total Quantity</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>Total Price</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Quantity</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Reusable % of Total</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>E1-0199</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2.00 pcs</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>18.00 pcs</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>900.00%</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>58.31999999999999</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>E2-0047</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>42.00 pcs</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>525.00%</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>99.95999999999999</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PC-1220</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>56.00 pcs</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>44.00 pcs</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>78.57%</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>8.052</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PM-1006-SS</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>12.00 pcs</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>46.65</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>88.00 pcs</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>733.33%</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>41.052</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>UA-1212</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>96.00 pcs</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2400.00%</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>46.656</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>E1-2530</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0.00 pcs</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>E2-0166</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>6.00 pcs</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>76.95</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>44.00 pcs</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>733.33%</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>67.71600000000001</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>E2-0177</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>76.95</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>42.00 pcs</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>525.00%</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>64.63800000000001</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>E2-0545</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>46.00 pcs</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1150.00%</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>135.24</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>E2-0154</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>6.00 pcs</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>44.00 pcs</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>733.33%</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>49.89600000000001</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>E2-0611</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>95.25</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>42.00 pcs</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>525.00%</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>80.01000000000001</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BE9-2513 (Clear)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>28.00 ft</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>838</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>8.00, 12.00 ft</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>71.43%</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>349.1666666666666</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>E9-2512 (Clear)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>24.00 ft</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>0.00 ft</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BE9-2511 (Clear)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>24.00 ft</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>497</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>0.00 ft</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BE9-2515 (Clear)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>12.00 ft</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Flush Filler</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>E9-2512</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
+      <c r="C53" s="2" t="n">
+        <v>527</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>12.00 ft</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>263.5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BE9-2514 (Clear)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>12.00 ft</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>444</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>12.00 ft</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>BE9-2578 (Clear)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>12.00 ft</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>264</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>12.00 ft</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>E9-2519 (Clear)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
         <is>
           <t>24.00 ft</t>
         </is>
       </c>
-      <c r="H34" s="2" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Two Piece Mullion Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>BE9-2511</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>24.00 ft</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="n">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Horizontal Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>BE9-2515</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>12.00 ft</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="n">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Head</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>BE9-2514</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>12.00 ft</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="n">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Thermal Sill Flashing</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>BE9-2578</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>12.00 ft</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="n">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Glass Stop (Use with BE9-2514, BE9-2515, BE9-2517)</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>E9-2519</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>24.00 ft</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="n">
+      <c r="C56" s="2" t="n">
         <v>85.05</v>
       </c>
-    </row>
-    <row r="40">
-      <c r="E40" s="1" t="inlineStr">
-        <is>
-          <t>GLASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="E41" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F41" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G41" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H41" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="E42" t="inlineStr">
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>0.00 ft</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t>Glass Area</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>83.75 sqft</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>879.375</v>
+      </c>
+      <c r="D57" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>59.75 sqft</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="n">
-        <v>627.375</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="E43" s="1" t="inlineStr">
-        <is>
-          <t>FABRICATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="E44" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F44" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G44" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H44" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="E45" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>Joints Fabrication Labor</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>24.00 joints</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="D58" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>24.00 joints</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="E46" s="1" t="inlineStr">
-        <is>
-          <t>GLAZING GASKET</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="E47" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F47" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G47" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H47" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Gasket</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>E2-0052</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Gasket (E2-0052)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
         <is>
           <t>224.00 ft</t>
         </is>
       </c>
-      <c r="H48" s="2" t="n">
+      <c r="C59" s="2" t="n">
         <v>405</v>
       </c>
-    </row>
-    <row r="49">
-      <c r="H49" s="1" t="inlineStr">
-        <is>
-          <t>SYSTEM TOTAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="H50" s="2" t="n">
-        <v>6471.625</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="H51" s="1" t="inlineStr">
-        <is>
-          <t>RUNNING GRAND TOTAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="H52" s="2" t="n">
-        <v>6471.625</v>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>276.00 ft</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>123.21%</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>223.56</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>REUSABLE GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>1841.766666666667</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>REUSABLE % OF RUNNING GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>35.18%</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added a Discount Grand Total
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H143"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>1149</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="37">
@@ -1181,7 +1181,7 @@
     </row>
     <row r="38">
       <c r="H38" s="2" t="n">
-        <v>3979.25625</v>
+        <v>3910.25625</v>
       </c>
     </row>
     <row r="39">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>111</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1905,7 +1905,7 @@
     <row r="74">
       <c r="E74" t="inlineStr">
         <is>
-          <t>Door (3' X 8')</t>
+          <t>Door (3' X 9')</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="H74" s="2" t="n">
-        <v>1350</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="75">
@@ -1931,1484 +1931,718 @@
     </row>
     <row r="76">
       <c r="H76" s="2" t="n">
-        <v>1419.65625</v>
+        <v>1689.65625</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="inlineStr">
-        <is>
-          <t>System Input</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>YES 45TU FRONT SET(OG)</t>
-        </is>
-      </c>
-      <c r="E77" s="1" t="inlineStr">
-        <is>
-          <t>PROFILES</t>
+      <c r="H77" s="1" t="inlineStr">
+        <is>
+          <t>RUNNING GRAND TOTAL</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="inlineStr">
-        <is>
-          <t>Finish</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Clear</t>
-        </is>
-      </c>
-      <c r="E78" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F78" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G78" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H78" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
+      <c r="H78" s="2" t="n">
+        <v>5599.9125</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="inlineStr">
-        <is>
-          <t>Elevation Type</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Sill/Jamb Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>BE9-2513</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>0.17 ft</t>
-        </is>
-      </c>
-      <c r="H79" s="2" t="n">
-        <v>0</v>
+      <c r="H79" s="1" t="inlineStr">
+        <is>
+          <t>DISCOUNTED TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>Total Count</t>
-        </is>
-      </c>
-      <c r="B80" t="n">
-        <v>1</v>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Sill/Jamb Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>BE9-2513</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>0.08 ft</t>
+          <t>Part Number / Description</t>
+        </is>
+      </c>
+      <c r="B80" s="1" t="inlineStr">
+        <is>
+          <t>Total Quantity</t>
+        </is>
+      </c>
+      <c r="C80" s="1" t="inlineStr">
+        <is>
+          <t>Total Price</t>
+        </is>
+      </c>
+      <c r="D80" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Quantity</t>
+        </is>
+      </c>
+      <c r="E80" s="1" t="inlineStr">
+        <is>
+          <t>Reusable % of Total</t>
+        </is>
+      </c>
+      <c r="F80" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Cost</t>
         </is>
       </c>
       <c r="H80" s="2" t="n">
-        <v>0</v>
+        <v>5039.92125</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="inlineStr">
-        <is>
-          <t>Bays Wide</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>1</v>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>E1-0199</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>16.00 pcs</t>
+        </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Flush Filler</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>E9-2512</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
+          <t>400.00%</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>51.84</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>E2-0047</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>46.00 pcs</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>1150.00%</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>109.48</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>PC-1220</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>16.00 pcs</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>84.00 pcs</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>525.00%</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>15.372</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>PM-1006-SS</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>6.00 pcs</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>46.65</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>94.00 pcs</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>1566.67%</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>43.851</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>UA-1212</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>92.00 pcs</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>1150.00%</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>44.712</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>E1-2530</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>0.00 pcs</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>E2-0166</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>0.00 pcs</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>0.00 pcs</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>E2-0177</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>76.95</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>46.00 pcs</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>1150.00%</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>70.79400000000001</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>E2-0545</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>46.00 pcs</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>1150.00%</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>135.24</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>E2-0154</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>0.00 pcs</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>0.00 pcs</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>E2-0611</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="n">
+        <v>95.25</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>46.00 pcs</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>1150.00%</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>87.63</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>BE9-2513 (Clear)</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>0.50 ft</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>23.50 ft</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>4700.00%</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>410.2708333333333</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>E9-2512 (Clear)</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
         <is>
           <t>0.00 ft</t>
         </is>
       </c>
-      <c r="H81" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="1" t="inlineStr">
-        <is>
-          <t>Bays Tall</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>1</v>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Two Piece Mullion Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>BE9-2511</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
+      <c r="C93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" t="inlineStr">
         <is>
           <t>0.00 ft</t>
         </is>
       </c>
-      <c r="H82" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="1" t="inlineStr">
-        <is>
-          <t>Opening Width</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>1</v>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Horizontal Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>BE9-2515</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>0.08 ft</t>
-        </is>
-      </c>
-      <c r="H83" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="1" t="inlineStr">
-        <is>
-          <t>Opening Height</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>1</v>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Head</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>BE9-2514</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>0.08 ft</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="1" t="inlineStr">
-        <is>
-          <t>Sq Ft per Type</t>
-        </is>
-      </c>
-      <c r="B85" t="n">
-        <v>0.006944444444444444</v>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Thermal Sill Flashing</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>BE9-2578</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>0.08 ft</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="1" t="inlineStr">
-        <is>
-          <t>Total Sq Ft</t>
-        </is>
-      </c>
-      <c r="B86" t="n">
-        <v>0.006944444444444444</v>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Glass Stop (Use with BE9-2514, BE9-2515, BE9-2517)</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>E9-2519</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>0.08 ft</t>
-        </is>
-      </c>
-      <c r="H86" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="1" t="inlineStr">
-        <is>
-          <t>Perimeter Ft</t>
-        </is>
-      </c>
-      <c r="B87" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="1" t="inlineStr">
-        <is>
-          <t>Total Perimeter Ft</t>
-        </is>
-      </c>
-      <c r="B88" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E88" s="1" t="inlineStr">
-        <is>
-          <t>ACCESSORIES</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="E89" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F89" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G89" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H89" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>End Dam For Sill Flashing</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>E1-0199</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>2.00 pcs</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Water Deflector</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>E2-0047</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>2.00 pcs</t>
-        </is>
-      </c>
-      <c r="H91" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>#12 x 1-1/4” PHSMS Type AB, Zinc Plated Steel, For Screw Spline Attachment</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>PC-1220</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>8.00 pcs</t>
-        </is>
-      </c>
-      <c r="H92" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93">
       <c r="E93" t="inlineStr">
         <is>
-          <t>#10-24 x 3/8” PHMS, Stainless Steel, For Attachment of Sill to Sill Flashing</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>PM-1006-SS</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>3.00 pcs</t>
-        </is>
-      </c>
-      <c r="H93" s="2" t="n">
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>BE9-2511 (Clear)</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>0.00 ft</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>0.00 ft</t>
+        </is>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>#12 x 3/4” UFHSMS Type A, Zinc Plated Steel For End Dam Attachment</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>UA-1212</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>4.00 pcs</t>
-        </is>
-      </c>
-      <c r="H94" s="2" t="n">
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>BE9-2515 (Clear)</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>0.17 ft</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="n">
+        <v>527</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>23.83 ft</t>
+        </is>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Setting Block Chair Use with E2-0177 Setting Block at Sill</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>E1-2530</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>2.00 pcs</t>
-        </is>
-      </c>
-      <c r="H95" s="2" t="n">
-        <v>9</v>
+          <t>14300.00%</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="n">
+        <v>523.3402777777778</v>
       </c>
     </row>
     <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>BE9-2514 (Clear)</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>0.17 ft</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="n">
+        <v>444</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>23.83 ft</t>
+        </is>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Side Block For Intermediate Vertical Shallow Pocket</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>E2-0166</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>0.00 pcs</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="n">
-        <v>0</v>
+          <t>14300.00%</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="n">
+        <v>440.9166666666667</v>
       </c>
     </row>
     <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>BE9-2578 (Clear)</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>0.17 ft</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="n">
+        <v>264</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>23.83 ft</t>
+        </is>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Setting Block For Sill</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>E2-0177</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>2.00 pcs</t>
-        </is>
-      </c>
-      <c r="H97" s="2" t="n">
-        <v>0</v>
+          <t>14300.00%</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>262.1666666666667</v>
       </c>
     </row>
     <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>E9-2519 (Clear)</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>0.17 ft</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="n">
+        <v>85.05</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>23.83 ft</t>
+        </is>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>1-1/8” “W” Side Block For Jamb</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>E2-0545</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>2.00 pcs</t>
-        </is>
-      </c>
-      <c r="H98" s="2" t="n">
-        <v>0</v>
+          <t>14300.00%</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="n">
+        <v>84.45937500000001</v>
       </c>
     </row>
     <row r="99">
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>1/2” “W” Side Block For Intermediate Vertical Deep Pocket</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>E2-0154</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>0.00 pcs</t>
-        </is>
-      </c>
-      <c r="H99" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Glass Area</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>0.12 sqft</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="n">
+        <v>1.3125</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Setting Block For Intermediate Horizontal</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>E2-0611</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>2.00 pcs</t>
-        </is>
-      </c>
-      <c r="H100" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Joints Fabrication Labor</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>8.00 joints</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="E101" s="1" t="inlineStr">
-        <is>
-          <t>GLASS</t>
-        </is>
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Gasket (E2-0052)</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1.33 ft</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="n">
+        <v>405</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>498.67 ft</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>37400.00%</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="n">
+        <v>403.92</v>
       </c>
     </row>
     <row r="102">
-      <c r="E102" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F102" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G102" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H102" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Door (3' X 7')</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1.00 pcs</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="n">
+        <v>1080</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>Glass Area</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Door (3' X 9')</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1.00 pcs</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="n">
+        <v>1620</v>
+      </c>
+      <c r="D103" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>0.06 sqft</t>
-        </is>
-      </c>
-      <c r="H103" s="2" t="n">
-        <v>0.65625</v>
-      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>FABRICATION</t>
-        </is>
+          <t>REUSABLE GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="n">
+        <v>2683.992819444445</v>
       </c>
     </row>
     <row r="105">
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F105" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G105" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H105" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>Joints Fabrication Labor</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>4.00 joints</t>
-        </is>
-      </c>
-      <c r="H106" s="2" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="E107" s="1" t="inlineStr">
-        <is>
-          <t>GLAZING GASKET</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="E108" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F108" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G108" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H108" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Gasket</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>E2-0052</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>0.67 ft</t>
-        </is>
-      </c>
-      <c r="H109" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="E110" s="1" t="inlineStr">
-        <is>
-          <t>DOOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="E111" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F111" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G111" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H111" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Door (3' X 9')</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="H112" s="2" t="n">
-        <v>1620</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="H113" s="1" t="inlineStr">
-        <is>
-          <t>SYSTEM TOTAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="H114" s="2" t="n">
-        <v>1689.65625</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="H115" s="1" t="inlineStr">
-        <is>
-          <t>RUNNING GRAND TOTAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="H116" s="2" t="n">
-        <v>7088.56875</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="1" t="inlineStr">
-        <is>
-          <t>Part Number / Description</t>
-        </is>
-      </c>
-      <c r="B117" s="1" t="inlineStr">
-        <is>
-          <t>Total Quantity</t>
-        </is>
-      </c>
-      <c r="C117" s="1" t="inlineStr">
-        <is>
-          <t>Total Price</t>
-        </is>
-      </c>
-      <c r="D117" s="1" t="inlineStr">
-        <is>
-          <t>Reusable Material Quantity</t>
-        </is>
-      </c>
-      <c r="E117" s="1" t="inlineStr">
-        <is>
-          <t>Reusable % of Total</t>
-        </is>
-      </c>
-      <c r="F117" s="1" t="inlineStr">
-        <is>
-          <t>Reusable Material Cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>E1-0199</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>6.00 pcs</t>
-        </is>
-      </c>
-      <c r="C118" s="2" t="n">
-        <v>64.8</v>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>14.00 pcs</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>233.33%</t>
-        </is>
-      </c>
-      <c r="F118" s="2" t="n">
-        <v>45.36</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>E2-0047</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>6.00 pcs</t>
-        </is>
-      </c>
-      <c r="C119" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>44.00 pcs</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>733.33%</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="n">
-        <v>104.72</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>PC-1220</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>24.00 pcs</t>
-        </is>
-      </c>
-      <c r="C120" s="2" t="n">
-        <v>18.3</v>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>76.00 pcs</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>316.67%</t>
-        </is>
-      </c>
-      <c r="F120" s="2" t="n">
-        <v>13.908</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>PM-1006-SS</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>9.00 pcs</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="n">
-        <v>46.65</v>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>91.00 pcs</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>1011.11%</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="n">
-        <v>42.4515</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>UA-1212</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>12.00 pcs</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="n">
-        <v>48.6</v>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>88.00 pcs</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>733.33%</t>
-        </is>
-      </c>
-      <c r="F122" s="2" t="n">
-        <v>42.768</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>E1-2530</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>6.00 pcs</t>
-        </is>
-      </c>
-      <c r="C123" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>0.00 pcs</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="F123" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>E2-0166</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>0.00 pcs</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>0.00 pcs</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="F124" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>E2-0177</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>6.00 pcs</t>
-        </is>
-      </c>
-      <c r="C125" s="2" t="n">
-        <v>76.95</v>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>44.00 pcs</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>733.33%</t>
-        </is>
-      </c>
-      <c r="F125" s="2" t="n">
-        <v>67.71600000000001</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>E2-0545</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>6.00 pcs</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="n">
-        <v>147</v>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>44.00 pcs</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>733.33%</t>
-        </is>
-      </c>
-      <c r="F126" s="2" t="n">
-        <v>129.36</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>E2-0154</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>0.00 pcs</t>
-        </is>
-      </c>
-      <c r="C127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>0.00 pcs</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="F127" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>E2-0611</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>6.00 pcs</t>
-        </is>
-      </c>
-      <c r="C128" s="2" t="n">
-        <v>95.25</v>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>44.00 pcs</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>733.33%</t>
-        </is>
-      </c>
-      <c r="F128" s="2" t="n">
-        <v>83.82000000000001</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>BE9-2513 (Clear)</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>0.75 ft</t>
-        </is>
-      </c>
-      <c r="C129" s="2" t="n">
-        <v>419</v>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>23.25 ft</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>3100.00%</t>
-        </is>
-      </c>
-      <c r="F129" s="2" t="n">
-        <v>405.90625</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>E9-2512 (Clear)</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>0.00 ft</t>
-        </is>
-      </c>
-      <c r="C130" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>0.00 ft</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="F130" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>BE9-2511 (Clear)</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>0.00 ft</t>
-        </is>
-      </c>
-      <c r="C131" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>0.00 ft</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="F131" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>BE9-2515 (Clear)</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>0.25 ft</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="n">
-        <v>527</v>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>23.75 ft</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>9500.00%</t>
-        </is>
-      </c>
-      <c r="F132" s="2" t="n">
-        <v>521.5104166666667</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>BE9-2514 (Clear)</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>0.25 ft</t>
-        </is>
-      </c>
-      <c r="C133" s="2" t="n">
-        <v>444</v>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>23.75 ft</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>9500.00%</t>
-        </is>
-      </c>
-      <c r="F133" s="2" t="n">
-        <v>439.3750000000001</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>BE9-2578 (Clear)</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>0.25 ft</t>
-        </is>
-      </c>
-      <c r="C134" s="2" t="n">
-        <v>264</v>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>23.75 ft</t>
-        </is>
-      </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>9500.00%</t>
-        </is>
-      </c>
-      <c r="F134" s="2" t="n">
-        <v>261.2500000000001</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>E9-2519 (Clear)</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>0.25 ft</t>
-        </is>
-      </c>
-      <c r="C135" s="2" t="n">
-        <v>85.05</v>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>23.75 ft</t>
-        </is>
-      </c>
-      <c r="E135" t="inlineStr">
-        <is>
-          <t>9500.00%</t>
-        </is>
-      </c>
-      <c r="F135" s="2" t="n">
-        <v>84.1640625</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>Glass Area</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>0.19 sqft</t>
-        </is>
-      </c>
-      <c r="C136" s="2" t="n">
-        <v>1.96875</v>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E136" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F136" s="2" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>Joints Fabrication Labor</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>12.00 joints</t>
-        </is>
-      </c>
-      <c r="C137" s="2" t="n">
-        <v>180</v>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E137" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F137" s="2" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>Gasket (E2-0052)</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>2.00 ft</t>
-        </is>
-      </c>
-      <c r="C138" s="2" t="n">
-        <v>405</v>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>498.00 ft</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>24900.00%</t>
-        </is>
-      </c>
-      <c r="F138" s="2" t="n">
-        <v>403.38</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>Door (3' X 7')</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="C139" s="2" t="n">
-        <v>1149</v>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E139" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F139" s="2" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>Door (3' X 8')</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="C140" s="2" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E140" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F140" s="2" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>Door (3' X 9')</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="C141" s="2" t="n">
-        <v>1620</v>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E141" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F141" s="2" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="E142" s="1" t="inlineStr">
-        <is>
-          <t>REUSABLE GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="F142" s="2" t="n">
-        <v>2645.689229166667</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="E143" s="1" t="inlineStr">
-        <is>
           <t>REUSABLE % OF RUNNING GRAND TOTAL</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>37.32%</t>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>47.93%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Door Refinement Exceeding Glass
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -430,7 +430,7 @@
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="76" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -506,7 +506,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.17 ft</t>
+          <t>16.00 ft</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -534,11 +534,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0</v>
+        <v>419</v>
       </c>
     </row>
     <row r="5">
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -562,11 +562,11 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -590,11 +590,11 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0</v>
+        <v>497</v>
       </c>
     </row>
     <row r="7">
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>144</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>96</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.006944444444444444</v>
+        <v>96</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -674,7 +674,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.006944444444444444</v>
+        <v>96</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -702,7 +702,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.3333333333333333</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12">
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.3333333333333333</v>
+        <v>40</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
@@ -742,10 +742,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1 x Narrow Door ($1,632.00)
-  with: Continuous Hinges, Electric Strike; 
-1 x Narrow Door ($1,632.00)
-  with: Exit Devices</t>
+          <t>1 x Narrow Door ($1,632.00)</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -802,7 +799,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -822,7 +819,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>56.00 pcs</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -842,7 +839,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3.00 pcs</t>
+          <t>12.00 pcs</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -882,11 +879,11 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20">
@@ -902,11 +899,11 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>0</v>
+        <v>76.95</v>
       </c>
     </row>
     <row r="21">
@@ -922,7 +919,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
@@ -942,7 +939,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
@@ -962,11 +959,11 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="24">
@@ -982,7 +979,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
@@ -1031,11 +1028,11 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0.00 sqft</t>
+          <t>62.75 sqft</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>0</v>
+        <v>658.875</v>
       </c>
     </row>
     <row r="28">
@@ -1080,7 +1077,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>42.00 sqft</t>
+          <t>21.00 sqft</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
@@ -1129,11 +1126,11 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>4.00 joints</t>
+          <t>24.00 joints</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>60</v>
+        <v>360</v>
       </c>
     </row>
     <row r="34">
@@ -1178,7 +1175,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0.67 ft</t>
+          <t>224.00 ft</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
@@ -1235,440 +1232,448 @@
       </c>
     </row>
     <row r="40">
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Door (3' X 7')</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="n">
-        <v>1632</v>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>SYSTEM TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="41">
-      <c r="H41" s="1" t="inlineStr">
-        <is>
-          <t>SYSTEM TOTAL</t>
-        </is>
+      <c r="H41" s="2" t="n">
+        <v>6647.125</v>
       </c>
     </row>
     <row r="42">
-      <c r="H42" s="2" t="n">
-        <v>6093.6</v>
+      <c r="H42" s="1" t="inlineStr">
+        <is>
+          <t>RUNNING GRAND TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="43">
-      <c r="H43" s="1" t="inlineStr">
-        <is>
-          <t>RUNNING GRAND TOTAL</t>
-        </is>
+      <c r="H43" s="2" t="n">
+        <v>6647.125</v>
       </c>
     </row>
     <row r="44">
-      <c r="H44" s="2" t="n">
-        <v>6093.6</v>
+      <c r="H44" s="1" t="inlineStr">
+        <is>
+          <t>DISCOUNTED TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="45">
-      <c r="H45" s="1" t="inlineStr">
-        <is>
-          <t>DISCOUNTED TOTAL</t>
-        </is>
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Part Number / Description</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>Total Quantity</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>Total Price</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Quantity</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Reusable % of Total</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Cost</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>5982.4125</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="inlineStr">
-        <is>
-          <t>Part Number / Description</t>
-        </is>
-      </c>
-      <c r="B46" s="1" t="inlineStr">
-        <is>
-          <t>Total Quantity</t>
-        </is>
-      </c>
-      <c r="C46" s="1" t="inlineStr">
-        <is>
-          <t>Total Price</t>
-        </is>
-      </c>
-      <c r="D46" s="1" t="inlineStr">
-        <is>
-          <t>Reusable Material Quantity</t>
-        </is>
-      </c>
-      <c r="E46" s="1" t="inlineStr">
-        <is>
-          <t>Reusable % of Total</t>
-        </is>
-      </c>
-      <c r="F46" s="1" t="inlineStr">
-        <is>
-          <t>Reusable Material Cost</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="n">
-        <v>5484.240000000001</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>E1-0199</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2.00 pcs</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>18.00 pcs</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>900.00%</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>58.31999999999999</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>E1-0199</t>
+          <t>E2-0047</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>64.8</v>
+        <v>119</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>18.00 pcs</t>
+          <t>42.00 pcs</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>900.00%</t>
+          <t>525.00%</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>58.31999999999999</v>
+        <v>99.95999999999999</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>E2-0047</t>
+          <t>PC-1220</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>56.00 pcs</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>119</v>
+        <v>18.3</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2400.00%</t>
+          <t>78.57%</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>114.24</v>
+        <v>8.052</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PC-1220</t>
+          <t>PM-1006-SS</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>12.00 pcs</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>18.3</v>
+        <v>46.65</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>92.00 pcs</t>
+          <t>88.00 pcs</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1150.00%</t>
+          <t>733.33%</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>16.836</v>
+        <v>41.052</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PM-1006-SS</t>
+          <t>UA-1212</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>3.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>46.65</v>
+        <v>48.6</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>97.00 pcs</t>
+          <t>96.00 pcs</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>3233.33%</t>
+          <t>2400.00%</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>45.2505</v>
+        <v>46.656</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>UA-1212</t>
+          <t>E1-2530</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>48.6</v>
+        <v>36</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>96.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2400.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>46.656</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>E1-2530</t>
+          <t>E2-0166</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>9</v>
+        <v>76.95</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>733.33%</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0</v>
+        <v>67.71600000000001</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>E2-0166</t>
+          <t>E2-0177</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>0</v>
+        <v>76.95</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>42.00 pcs</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>525.00%</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0</v>
+        <v>64.63800000000001</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>E2-0177</t>
+          <t>E2-0545</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>76.95</v>
+        <v>147</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>46.00 pcs</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2400.00%</t>
+          <t>1150.00%</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>73.87200000000001</v>
+        <v>135.24</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>E2-0545</t>
+          <t>E2-0154</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>147</v>
+        <v>56.7</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2400.00%</t>
+          <t>733.33%</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>141.12</v>
+        <v>49.89600000000001</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>E2-0154</t>
+          <t>E2-0611</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>0</v>
+        <v>95.25</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>42.00 pcs</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>525.00%</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0</v>
+        <v>80.01000000000001</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>E2-0611</t>
+          <t>BE9-2513 (Clear)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>28.00 ft</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>95.25</v>
+        <v>838</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>8.00, 12.00 ft</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2400.00%</t>
+          <t>71.43%</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>91.44</v>
+        <v>349.1666666666666</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BE9-2513 (Clear)</t>
+          <t>E9-2512 (Clear)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>0.25 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>419</v>
+        <v>150</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>23.75 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>9500.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>414.6354166666666</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>E9-2512 (Clear)</t>
+          <t>BE9-2511 (Clear)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>0</v>
+        <v>497</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1687,152 +1692,150 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BE9-2511 (Clear)</t>
+          <t>BE9-2515 (Clear)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>0</v>
+        <v>527</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0</v>
+        <v>263.5</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BE9-2515 (Clear)</t>
+          <t>BE9-2514 (Clear)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>527</v>
+        <v>444</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>23.92 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>28700.00%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>525.1701388888889</v>
+        <v>222</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BE9-2514 (Clear)</t>
+          <t>BE9-2578 (Clear)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>444</v>
+        <v>264</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>23.92 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>28700.00%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>442.4583333333334</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BE9-2578 (Clear)</t>
+          <t>E9-2519 (Clear)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>264</v>
+        <v>85.05</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>23.92 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>28700.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>263.0833333333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>E9-2519 (Clear)</t>
+          <t>Glass Area (Adjusted)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>62.75 sqft</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>85.05</v>
+        <v>658.875</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>23.92 ft</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>28700.00%</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="n">
-        <v>84.7546875</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Glass Area (Adjusted)</t>
+          <t>Door Area (to subtract from glass)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>0.00 sqft</t>
+          <t>21.00 sqft</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -1853,16 +1856,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Door Area (to subtract from glass)</t>
+          <t>Joints Fabrication Labor</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>42.00 sqft</t>
+          <t>24.00 joints</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -1879,102 +1882,76 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Joints Fabrication Labor</t>
+          <t>Gasket (E2-0052)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>4.00 joints</t>
+          <t>224.00 ft</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>60</v>
+        <v>405</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr"/>
+          <t>276.00 ft</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>123.21%</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>223.56</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Gasket (E2-0052)</t>
+          <t>Door (3' X 7')</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>0.67 ft</t>
+          <t>1.00 pcs</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>405</v>
+        <v>1632</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>499.33 ft</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>74900.00%</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="n">
-        <v>404.46</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Door (3' X 7')</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>2.00 pcs</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="n">
-        <v>3264</v>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr"/>
+      <c r="E69" s="1" t="inlineStr">
+        <is>
+          <t>REUSABLE GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>1841.766666666667</v>
+      </c>
     </row>
     <row r="70">
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>REUSABLE GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="n">
-        <v>2722.296409722223</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="E71" s="1" t="inlineStr">
-        <is>
           <t>REUSABLE % OF RUNNING GRAND TOTAL</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>44.67%</t>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>27.71%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GOt Discount, still need to fix list int error
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -426,7 +426,7 @@
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="76" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>419</v>
+        <v>244.696</v>
       </c>
     </row>
     <row r="4">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>527</v>
+        <v>307.768</v>
       </c>
     </row>
     <row r="8">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>444</v>
+        <v>259.296</v>
       </c>
     </row>
     <row r="9">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>264</v>
+        <v>154.176</v>
       </c>
     </row>
     <row r="10">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>85.05</v>
+        <v>49.6692</v>
       </c>
     </row>
     <row r="11">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>64.8</v>
+        <v>37.8432</v>
       </c>
     </row>
     <row r="15">
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>119</v>
+        <v>69.496</v>
       </c>
     </row>
     <row r="16">
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>18.3</v>
+        <v>10.6872</v>
       </c>
     </row>
     <row r="17">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46.65</v>
+        <v>27.2436</v>
       </c>
     </row>
     <row r="18">
@@ -863,7 +863,7 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>48.6</v>
+        <v>28.3824</v>
       </c>
     </row>
     <row r="19">
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>9</v>
+        <v>5.255999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>76.95</v>
+        <v>44.9388</v>
       </c>
     </row>
     <row r="22">
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>147</v>
+        <v>85.848</v>
       </c>
     </row>
     <row r="23">
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>95.25</v>
+        <v>55.626</v>
       </c>
     </row>
     <row r="25">
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>405</v>
+        <v>236.52</v>
       </c>
     </row>
     <row r="37">
@@ -1191,7 +1191,7 @@
     </row>
     <row r="38">
       <c r="H38" s="2" t="n">
-        <v>2830.25625</v>
+        <v>1678.10265</v>
       </c>
     </row>
     <row r="39">
@@ -1203,7 +1203,7 @@
     </row>
     <row r="40">
       <c r="H40" s="2" t="n">
-        <v>2830.25625</v>
+        <v>1678.10265</v>
       </c>
     </row>
     <row r="41">
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="H42" s="2" t="n">
-        <v>2547.230625</v>
+        <v>1510.292385</v>
       </c>
     </row>
     <row r="43">
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>64.8</v>
+        <v>37.8432</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>58.31999999999999</v>
+        <v>34.05887999999999</v>
       </c>
     </row>
     <row r="44">
@@ -1288,7 +1288,7 @@
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>119</v>
+        <v>69.496</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>114.24</v>
+        <v>66.71615999999999</v>
       </c>
     </row>
     <row r="45">
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>18.3</v>
+        <v>10.6872</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>16.836</v>
+        <v>9.832223999999998</v>
       </c>
     </row>
     <row r="46">
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>46.65</v>
+        <v>27.2436</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>45.2505</v>
+        <v>26.426292</v>
       </c>
     </row>
     <row r="47">
@@ -1372,7 +1372,7 @@
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>48.6</v>
+        <v>28.3824</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46.656</v>
+        <v>27.247104</v>
       </c>
     </row>
     <row r="48">
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>9</v>
+        <v>5.255999999999999</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1456,7 +1456,7 @@
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>76.95</v>
+        <v>44.9388</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>73.87200000000001</v>
+        <v>43.141248</v>
       </c>
     </row>
     <row r="51">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>147</v>
+        <v>85.848</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>141.12</v>
+        <v>82.41408</v>
       </c>
     </row>
     <row r="52">
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>95.25</v>
+        <v>55.626</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>91.44</v>
+        <v>53.40096</v>
       </c>
     </row>
     <row r="54">
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>419</v>
+        <v>244.696</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1581,7 +1581,7 @@
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>414.6354166666666</v>
+        <v>242.1470833333333</v>
       </c>
     </row>
     <row r="55">
@@ -1652,7 +1652,7 @@
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>527</v>
+        <v>307.768</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>525.1701388888889</v>
+        <v>306.6993611111111</v>
       </c>
     </row>
     <row r="58">
@@ -1680,7 +1680,7 @@
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>444</v>
+        <v>259.296</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>442.4583333333334</v>
+        <v>258.3956666666667</v>
       </c>
     </row>
     <row r="59">
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>264</v>
+        <v>154.176</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>263.0833333333334</v>
+        <v>153.6406666666667</v>
       </c>
     </row>
     <row r="60">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>85.05</v>
+        <v>49.6692</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>84.7546875</v>
+        <v>49.4967375</v>
       </c>
     </row>
     <row r="61">
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>0.041015625</v>
+        <v>0.65625</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>405</v>
+        <v>236.52</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>404.46</v>
+        <v>236.20464</v>
       </c>
     </row>
     <row r="65">
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>2722.296409722223</v>
+        <v>1589.821103277778</v>
       </c>
     </row>
     <row r="66">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>96.19%</t>
+          <t>94.74%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed percentage on waste
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -772,8 +772,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1 x Narrow Door ($2,425.25)
-  with: Electric Strike</t>
+          <t>None</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -1102,14 +1101,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>41.75 sqft</t>
+          <t>83.75 sqft</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>438.375</v>
+        <v>879.375</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>438.375</v>
+        <v>879.375</v>
       </c>
     </row>
     <row r="28">
@@ -1159,7 +1158,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>42.00 sqft</t>
+          <t>0.00 sqft</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
@@ -1284,337 +1283,373 @@
       </c>
     </row>
     <row r="37">
-      <c r="E37" s="1" t="inlineStr">
-        <is>
-          <t>DOOR</t>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>ORIGINAL SYSTEM TOTAL</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="E38" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F38" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G38" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H38" s="1" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
-      <c r="I38" s="1" t="inlineStr">
-        <is>
-          <t>Discounted Price</t>
-        </is>
+      <c r="I38" s="2" t="n">
+        <v>5235.625</v>
       </c>
     </row>
     <row r="39">
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Door (6' X 7')</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="n">
-        <v>2425.25</v>
-      </c>
-      <c r="I39" s="2" t="n">
-        <v>2425.25</v>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>DISCOUNTED SYSTEM TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="40">
-      <c r="I40" s="1" t="inlineStr">
-        <is>
-          <t>ORIGINAL SYSTEM TOTAL</t>
-        </is>
+      <c r="I40" s="2" t="n">
+        <v>3573.185</v>
       </c>
     </row>
     <row r="41">
-      <c r="I41" s="2" t="n">
-        <v>7219.875</v>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>ORIGINAL RUNNING GRAND TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="42">
-      <c r="I42" s="1" t="inlineStr">
-        <is>
-          <t>DISCOUNTED SYSTEM TOTAL</t>
-        </is>
+      <c r="I42" s="2" t="n">
+        <v>5235.625</v>
       </c>
     </row>
     <row r="43">
-      <c r="I43" s="2" t="n">
-        <v>5557.434999999999</v>
+      <c r="I43" s="1" t="inlineStr">
+        <is>
+          <t>RUNNING GRAND TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="44">
-      <c r="I44" s="1" t="inlineStr">
-        <is>
-          <t>ORIGINAL RUNNING GRAND TOTAL</t>
-        </is>
+      <c r="I44" s="2" t="n">
+        <v>3573.185</v>
       </c>
     </row>
     <row r="45">
-      <c r="I45" s="2" t="n">
-        <v>7219.875</v>
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Part Number / Description</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>Total Quantity</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>Original Total Price</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>Discounted Total Price</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Quantity</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>Reusable % of Total</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Cost</t>
+        </is>
       </c>
     </row>
     <row r="46">
-      <c r="I46" s="1" t="inlineStr">
-        <is>
-          <t>RUNNING GRAND TOTAL</t>
-        </is>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>E1-0199</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2.00 pcs</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>37.8432</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>18.00 pcs</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>90.00%</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>34.05887999999999</v>
       </c>
     </row>
     <row r="47">
-      <c r="I47" s="2" t="n">
-        <v>5557.434999999999</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>E2-0047</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>69.496</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>42.00 pcs</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>84.00%</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>58.37663999999999</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="inlineStr">
-        <is>
-          <t>Part Number / Description</t>
-        </is>
-      </c>
-      <c r="B48" s="1" t="inlineStr">
-        <is>
-          <t>Total Quantity</t>
-        </is>
-      </c>
-      <c r="C48" s="1" t="inlineStr">
-        <is>
-          <t>Original Total Price</t>
-        </is>
-      </c>
-      <c r="D48" s="1" t="inlineStr">
-        <is>
-          <t>Discounted Total Price</t>
-        </is>
-      </c>
-      <c r="E48" s="1" t="inlineStr">
-        <is>
-          <t>Reusable Material Quantity</t>
-        </is>
-      </c>
-      <c r="F48" s="1" t="inlineStr">
-        <is>
-          <t>Reusable % of Total</t>
-        </is>
-      </c>
-      <c r="G48" s="1" t="inlineStr">
-        <is>
-          <t>Reusable Material Cost</t>
-        </is>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PC-1220</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>56.00 pcs</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>10.6872</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>44.00 pcs</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>44.00%</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>4.702368</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>E1-0199</t>
+          <t>PM-1006-SS</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>12.00 pcs</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>64.8</v>
+        <v>46.65</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>37.8432</v>
+        <v>27.2436</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>18.00 pcs</t>
+          <t>88.00 pcs</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>900.00%</t>
+          <t>88.00%</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>34.05887999999999</v>
+        <v>23.974368</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>E2-0047</t>
+          <t>UA-1212</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>119</v>
+        <v>48.6</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>69.496</v>
+        <v>28.3824</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>42.00 pcs</t>
+          <t>96.00 pcs</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>525.00%</t>
+          <t>96.00%</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>58.37663999999999</v>
+        <v>27.247104</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PC-1220</t>
+          <t>E1-2530</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>56.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>18.3</v>
+        <v>36</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>10.6872</v>
+        <v>21.024</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>44.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>78.57%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>4.702368</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PM-1006-SS</t>
+          <t>E2-0166</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>12.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>46.65</v>
+        <v>76.95</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>27.2436</v>
+        <v>44.9388</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>88.00 pcs</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>733.33%</t>
+          <t>88.00%</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>23.974368</v>
+        <v>39.54614400000001</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>UA-1212</t>
+          <t>E2-0177</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>48.6</v>
+        <v>76.95</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>28.3824</v>
+        <v>44.9388</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>96.00 pcs</t>
+          <t>42.00 pcs</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2400.00%</t>
+          <t>84.00%</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>27.247104</v>
+        <v>37.748592</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>E1-2530</t>
+          <t>E2-0545</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>36</v>
+        <v>147</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>21.024</v>
+        <v>85.848</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>46.00 pcs</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>92.00%</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0</v>
+        <v>78.98016</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>E2-0166</t>
+          <t>E2-0154</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,10 +1658,10 @@
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>76.95</v>
+        <v>56.7</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>44.9388</v>
+        <v>33.1128</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1635,17 +1670,17 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>733.33%</t>
+          <t>88.00%</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>39.54614400000001</v>
+        <v>29.139264</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>E2-0177</t>
+          <t>E2-0611</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1654,10 +1689,10 @@
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>76.95</v>
+        <v>95.25</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>44.9388</v>
+        <v>55.626</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1666,487 +1701,365 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>525.00%</t>
+          <t>84.00%</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>37.748592</v>
+        <v>46.72584</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>E2-0545</t>
+          <t>BE9-2513 (Clear)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>28.00 ft</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>147</v>
+        <v>838</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>85.848</v>
+        <v>489.392</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>46.00 pcs</t>
+          <t>8.00, 12.00 ft</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>1150.00%</t>
+          <t>41.67%</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>78.98016</v>
+        <v>203.9133333333333</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>E2-0154</t>
+          <t>E9-2512 (Clear)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>6.00 pcs</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>56.7</v>
+        <v>150</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>33.1128</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>44.00 pcs</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>733.33%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>29.139264</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>E2-0611</t>
+          <t>BE9-2511 (Clear)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>95.25</v>
+        <v>497</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>55.626</v>
+        <v>290.248</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>42.00 pcs</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>525.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>46.72584</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BE9-2513 (Clear)</t>
+          <t>BE9-2515 (Clear)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>28.00 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>838</v>
+        <v>527</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>489.392</v>
+        <v>307.768</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>8.00, 12.00 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>71.43%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>203.9133333333333</v>
+        <v>153.884</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>E9-2512 (Clear)</t>
+          <t>BE9-2514 (Clear)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>24.00 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>150</v>
+        <v>444</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>87.59999999999999</v>
+        <v>259.296</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0</v>
+        <v>129.648</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BE9-2511 (Clear)</t>
+          <t>BE9-2578 (Clear)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>24.00 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>497</v>
+        <v>264</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>290.248</v>
+        <v>154.176</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>12.00 ft</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0</v>
+        <v>77.08799999999999</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BE9-2515 (Clear)</t>
+          <t>E9-2519 (Clear)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>527</v>
+        <v>85.05</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>307.768</v>
+        <v>49.6692</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>153.884</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BE9-2514 (Clear)</t>
+          <t>Glass Area (Adjusted)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>83.75 sqft</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>444</v>
+        <v>0</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>259.296</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="n">
-        <v>129.648</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BE9-2578 (Clear)</t>
+          <t>Door Area (to subtract from glass)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>0.00 sqft</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>154.176</v>
+        <v>0</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="n">
-        <v>77.08799999999999</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>E9-2519 (Clear)</t>
+          <t>Joints Fabrication Labor</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>24.00 ft</t>
+          <t>24.00 joints</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>85.05</v>
+        <v>0</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>49.6692</v>
+        <v>0</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Glass Area (Adjusted)</t>
+          <t>Gasket (E2-0052)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>41.75 sqft</t>
+          <t>224.00 ft</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>0</v>
+        <v>405</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0</v>
+        <v>236.52</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr"/>
+          <t>276.00 ft</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>55.20%</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>130.55904</v>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Door Area (to subtract from glass)</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>42.00 sqft</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr"/>
+      <c r="F68" s="1" t="inlineStr">
+        <is>
+          <t>REUSABLE GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>1075.591733333333</v>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Joints Fabrication Labor</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>24.00 joints</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Gasket (E2-0052)</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>224.00 ft</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="n">
-        <v>405</v>
-      </c>
-      <c r="D70" s="2" t="n">
-        <v>236.52</v>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>276.00 ft</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>123.21%</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="n">
-        <v>130.55904</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Door (6' X 7')</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="F72" s="1" t="inlineStr">
-        <is>
-          <t>REUSABLE GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="n">
-        <v>1075.591733333333</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="F73" s="1" t="inlineStr">
+      <c r="F69" s="1" t="inlineStr">
         <is>
           <t>REUSABLE % OF DISCOUNTED GRAND TOTAL</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>46.09%</t>
         </is>

</xml_diff>

<commit_message>
Added Glass Add back to Door Framing
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -431,7 +431,7 @@
     <col width="76" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -512,7 +512,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>16.00 ft</t>
+          <t>13.83 ft</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -543,14 +543,14 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>419</v>
+        <v>0</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>244.696</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -574,14 +574,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>24.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>87.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -605,14 +605,14 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>24.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>497</v>
+        <v>0</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>290.248</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>144</v>
+        <v>36</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -636,7 +636,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>96</v>
+        <v>20.75</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>96</v>
+        <v>20.75</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>24.00 ft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>40</v>
+        <v>19.83333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>40</v>
+        <v>19.83333333333334</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>1 x Narrow Door ($880.00)</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -860,7 +860,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>56.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -883,7 +883,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>12.00 pcs</t>
+          <t>3.00 pcs</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -929,14 +929,14 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>21.024</v>
+        <v>5.255999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -952,14 +952,14 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>6.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>76.95</v>
+        <v>0</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>44.9388</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -975,7 +975,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
@@ -998,7 +998,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
@@ -1021,14 +1021,14 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>6.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>56.7</v>
+        <v>0</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>33.1128</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
@@ -1101,14 +1101,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>83.75 sqft</t>
+          <t>11.78 sqft</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>879.375</v>
+        <v>123.6433333333334</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>879.375</v>
+        <v>123.6433333333334</v>
       </c>
     </row>
     <row r="28">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0.00 sqft</t>
+          <t>21.00 sqft</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
@@ -1215,14 +1215,14 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>24.00 joints</t>
+          <t>4.00 joints</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>360</v>
+        <v>60</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>360</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>224.00 ft</t>
+          <t>39.67 ft</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
@@ -1283,234 +1283,198 @@
       </c>
     </row>
     <row r="37">
-      <c r="I37" s="1" t="inlineStr">
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>DOOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>Original Price</t>
+        </is>
+      </c>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>Discounted Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Door (3' X 7')</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>1.00 pcs</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>880</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="I40" s="1" t="inlineStr">
         <is>
           <t>ORIGINAL SYSTEM TOTAL</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="I38" s="2" t="n">
-        <v>5235.625</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="I39" s="1" t="inlineStr">
+    <row r="41">
+      <c r="I41" s="2" t="n">
+        <v>3833.243333333333</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="I42" s="1" t="inlineStr">
         <is>
           <t>DISCOUNTED SYSTEM TOTAL</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="I40" s="2" t="n">
-        <v>3573.185</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="I41" s="1" t="inlineStr">
+    <row r="43">
+      <c r="I43" s="2" t="n">
+        <v>2681.089733333333</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="I44" s="1" t="inlineStr">
         <is>
           <t>ORIGINAL RUNNING GRAND TOTAL</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="I42" s="2" t="n">
-        <v>5235.625</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="I43" s="1" t="inlineStr">
+    <row r="45">
+      <c r="I45" s="2" t="n">
+        <v>3833.243333333333</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="I46" s="1" t="inlineStr">
         <is>
           <t>RUNNING GRAND TOTAL</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="I44" s="2" t="n">
-        <v>3573.185</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="inlineStr">
+    <row r="47">
+      <c r="I47" s="2" t="n">
+        <v>2681.089733333333</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>Part Number / Description</t>
         </is>
       </c>
-      <c r="B45" s="1" t="inlineStr">
+      <c r="B48" s="1" t="inlineStr">
         <is>
           <t>Total Quantity</t>
         </is>
       </c>
-      <c r="C45" s="1" t="inlineStr">
+      <c r="C48" s="1" t="inlineStr">
         <is>
           <t>Original Total Price</t>
         </is>
       </c>
-      <c r="D45" s="1" t="inlineStr">
+      <c r="D48" s="1" t="inlineStr">
         <is>
           <t>Discounted Total Price</t>
         </is>
       </c>
-      <c r="E45" s="1" t="inlineStr">
+      <c r="E48" s="1" t="inlineStr">
         <is>
           <t>Reusable Material Quantity</t>
         </is>
       </c>
-      <c r="F45" s="1" t="inlineStr">
+      <c r="F48" s="1" t="inlineStr">
         <is>
           <t>Reusable % of Total</t>
         </is>
       </c>
-      <c r="G45" s="1" t="inlineStr">
+      <c r="G48" s="1" t="inlineStr">
         <is>
           <t>Reusable Material Cost</t>
         </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>E1-0199</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>2.00 pcs</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="n">
-        <v>64.8</v>
-      </c>
-      <c r="D46" s="2" t="n">
-        <v>37.8432</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>18.00 pcs</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>90.00%</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="n">
-        <v>34.05887999999999</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>E2-0047</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>8.00 pcs</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="D47" s="2" t="n">
-        <v>69.496</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>42.00 pcs</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>84.00%</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="n">
-        <v>58.37663999999999</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>PC-1220</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>56.00 pcs</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>18.3</v>
-      </c>
-      <c r="D48" s="2" t="n">
-        <v>10.6872</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>44.00 pcs</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>44.00%</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="n">
-        <v>4.702368</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PM-1006-SS</t>
+          <t>E1-0199</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>12.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>46.65</v>
+        <v>64.8</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>27.2436</v>
+        <v>37.8432</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>88.00 pcs</t>
+          <t>18.00 pcs</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>88.00%</t>
+          <t>90.00%</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>23.974368</v>
+        <v>34.05887999999999</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>UA-1212</t>
+          <t>E2-0047</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>48.6</v>
+        <v>119</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>28.3824</v>
+        <v>69.496</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>96.00 pcs</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -1519,13 +1483,13 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>27.247104</v>
+        <v>66.71615999999999</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>E1-2530</t>
+          <t>PC-1220</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1534,231 +1498,231 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>36</v>
+        <v>18.3</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>21.024</v>
+        <v>10.6872</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>92.00 pcs</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>92.00%</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0</v>
+        <v>9.832223999999998</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>E2-0166</t>
+          <t>PM-1006-SS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>6.00 pcs</t>
+          <t>3.00 pcs</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>76.95</v>
+        <v>46.65</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>44.9388</v>
+        <v>27.2436</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>44.00 pcs</t>
+          <t>97.00 pcs</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>88.00%</t>
+          <t>97.00%</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>39.54614400000001</v>
+        <v>26.426292</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>E2-0177</t>
+          <t>UA-1212</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>76.95</v>
+        <v>48.6</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>44.9388</v>
+        <v>28.3824</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>42.00 pcs</t>
+          <t>96.00 pcs</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>84.00%</t>
+          <t>96.00%</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>37.748592</v>
+        <v>27.247104</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>E2-0545</t>
+          <t>E1-2530</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>147</v>
+        <v>9</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>85.848</v>
+        <v>5.255999999999999</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>46.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>92.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>78.98016</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>E2-0154</t>
+          <t>E2-0166</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>56.7</v>
+        <v>0</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>33.1128</v>
+        <v>0</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>44.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>88.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>29.139264</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>E2-0611</t>
+          <t>E2-0177</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>95.25</v>
+        <v>76.95</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>55.626</v>
+        <v>44.9388</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>42.00 pcs</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>84.00%</t>
+          <t>96.00%</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>46.72584</v>
+        <v>43.141248</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BE9-2513 (Clear)</t>
+          <t>E2-0545</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>28.00 ft</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>838</v>
+        <v>147</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>489.392</v>
+        <v>85.848</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>8.00, 12.00 ft</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>41.67%</t>
+          <t>96.00%</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>203.9133333333333</v>
+        <v>82.41408</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>E9-2512 (Clear)</t>
+          <t>E2-0154</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>24.00 ft</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>87.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -1773,295 +1737,417 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BE9-2511 (Clear)</t>
+          <t>E2-0611</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>24.00 ft</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>497</v>
+        <v>95.25</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>290.248</v>
+        <v>55.626</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>96.00%</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0</v>
+        <v>53.40096</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BE9-2515 (Clear)</t>
+          <t>BE9-2513 (Clear)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>16.83 ft</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>527</v>
+        <v>419</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>307.768</v>
+        <v>244.696</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>7.17 ft</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>29.86%</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>153.884</v>
+        <v>73.06894444444443</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BE9-2514 (Clear)</t>
+          <t>E9-2512 (Clear)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>444</v>
+        <v>0</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>259.296</v>
+        <v>0</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>129.648</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BE9-2578 (Clear)</t>
+          <t>BE9-2511 (Clear)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>154.176</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>77.08799999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>E9-2519 (Clear)</t>
+          <t>BE9-2515 (Clear)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>24.00 ft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>85.05</v>
+        <v>527</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>49.6692</v>
+        <v>307.768</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>21.00 ft</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>87.50%</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0</v>
+        <v>269.297</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Glass Area (Adjusted)</t>
+          <t>BE9-2514 (Clear)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>83.75 sqft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>0</v>
+        <v>444</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>0</v>
+        <v>259.296</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr"/>
+          <t>21.00 ft</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>87.50%</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>226.884</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Door Area (to subtract from glass)</t>
+          <t>BE9-2578 (Clear)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>0.00 sqft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0</v>
+        <v>154.176</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="inlineStr"/>
+          <t>21.00 ft</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>87.50%</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>134.904</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Joints Fabrication Labor</t>
+          <t>E9-2519 (Clear)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>24.00 joints</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>0</v>
+        <v>85.05</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0</v>
+        <v>49.6692</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr"/>
+          <t>21.00 ft</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>87.50%</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>43.46054999999999</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>Glass Area (Adjusted)</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>11.78 sqft</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Door Area (to subtract from glass)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>21.00 sqft</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Joints Fabrication Labor</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>4.00 joints</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
           <t>Gasket (E2-0052)</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>224.00 ft</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="n">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>39.67 ft</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="n">
         <v>405</v>
       </c>
-      <c r="D67" s="2" t="n">
+      <c r="D70" s="2" t="n">
         <v>236.52</v>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>276.00 ft</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>55.20%</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="n">
-        <v>130.55904</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="F68" s="1" t="inlineStr">
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>460.33 ft</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>92.07%</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>217.75608</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Door (3' X 7')</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1.00 pcs</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="F72" s="1" t="inlineStr">
         <is>
           <t>REUSABLE GRAND TOTAL</t>
         </is>
       </c>
-      <c r="G68" s="2" t="n">
-        <v>1075.591733333333</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="F69" s="1" t="inlineStr">
+      <c r="G72" s="2" t="n">
+        <v>1308.607522444444</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="F73" s="1" t="inlineStr">
         <is>
           <t>REUSABLE % OF DISCOUNTED GRAND TOTAL</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>46.09%</t>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>80.91%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Doors Addition with Glass Add back
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -772,7 +772,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1 x Narrow Door ($880.00)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -1101,14 +1101,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>11.78 sqft</t>
+          <t>17.56 sqft</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>123.6433333333334</v>
+        <v>184.3333333333333</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>123.6433333333334</v>
+        <v>184.3333333333333</v>
       </c>
     </row>
     <row r="28">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>21.00 sqft</t>
+          <t>0.00 sqft</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
@@ -1283,198 +1283,234 @@
       </c>
     </row>
     <row r="37">
-      <c r="E37" s="1" t="inlineStr">
-        <is>
-          <t>DOOR</t>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>ORIGINAL SYSTEM TOTAL</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="E38" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F38" s="1" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G38" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H38" s="1" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
-      <c r="I38" s="1" t="inlineStr">
-        <is>
-          <t>Discounted Price</t>
-        </is>
+      <c r="I38" s="2" t="n">
+        <v>3013.933333333333</v>
       </c>
     </row>
     <row r="39">
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Door (3' X 7')</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="n">
-        <v>880</v>
-      </c>
-      <c r="I39" s="2" t="n">
-        <v>880</v>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>DISCOUNTED SYSTEM TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="40">
-      <c r="I40" s="1" t="inlineStr">
-        <is>
-          <t>ORIGINAL SYSTEM TOTAL</t>
-        </is>
+      <c r="I40" s="2" t="n">
+        <v>1861.779733333333</v>
       </c>
     </row>
     <row r="41">
-      <c r="I41" s="2" t="n">
-        <v>3833.243333333333</v>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>ORIGINAL RUNNING GRAND TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="42">
-      <c r="I42" s="1" t="inlineStr">
-        <is>
-          <t>DISCOUNTED SYSTEM TOTAL</t>
-        </is>
+      <c r="I42" s="2" t="n">
+        <v>3013.933333333333</v>
       </c>
     </row>
     <row r="43">
-      <c r="I43" s="2" t="n">
-        <v>2681.089733333333</v>
+      <c r="I43" s="1" t="inlineStr">
+        <is>
+          <t>RUNNING GRAND TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="44">
-      <c r="I44" s="1" t="inlineStr">
-        <is>
-          <t>ORIGINAL RUNNING GRAND TOTAL</t>
-        </is>
+      <c r="I44" s="2" t="n">
+        <v>1861.779733333333</v>
       </c>
     </row>
     <row r="45">
-      <c r="I45" s="2" t="n">
-        <v>3833.243333333333</v>
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Part Number / Description</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>Total Quantity</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>Original Total Price</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>Discounted Total Price</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Quantity</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>Reusable % of Total</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>Reusable Material Cost</t>
+        </is>
       </c>
     </row>
     <row r="46">
-      <c r="I46" s="1" t="inlineStr">
-        <is>
-          <t>RUNNING GRAND TOTAL</t>
-        </is>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>E1-0199</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2.00 pcs</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>37.8432</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>18.00 pcs</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>90.00%</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>34.05887999999999</v>
       </c>
     </row>
     <row r="47">
-      <c r="I47" s="2" t="n">
-        <v>2681.089733333333</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>E2-0047</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2.00 pcs</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>69.496</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>48.00 pcs</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>96.00%</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>66.71615999999999</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="inlineStr">
-        <is>
-          <t>Part Number / Description</t>
-        </is>
-      </c>
-      <c r="B48" s="1" t="inlineStr">
-        <is>
-          <t>Total Quantity</t>
-        </is>
-      </c>
-      <c r="C48" s="1" t="inlineStr">
-        <is>
-          <t>Original Total Price</t>
-        </is>
-      </c>
-      <c r="D48" s="1" t="inlineStr">
-        <is>
-          <t>Discounted Total Price</t>
-        </is>
-      </c>
-      <c r="E48" s="1" t="inlineStr">
-        <is>
-          <t>Reusable Material Quantity</t>
-        </is>
-      </c>
-      <c r="F48" s="1" t="inlineStr">
-        <is>
-          <t>Reusable % of Total</t>
-        </is>
-      </c>
-      <c r="G48" s="1" t="inlineStr">
-        <is>
-          <t>Reusable Material Cost</t>
-        </is>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PC-1220</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>10.6872</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>92.00 pcs</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>92.00%</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>9.832223999999998</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>E1-0199</t>
+          <t>PM-1006-SS</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>3.00 pcs</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>64.8</v>
+        <v>46.65</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>37.8432</v>
+        <v>27.2436</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>18.00 pcs</t>
+          <t>97.00 pcs</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>90.00%</t>
+          <t>97.00%</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>34.05887999999999</v>
+        <v>26.426292</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>E2-0047</t>
+          <t>UA-1212</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>119</v>
+        <v>48.6</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>69.496</v>
+        <v>28.3824</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>96.00 pcs</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -1483,91 +1519,91 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>66.71615999999999</v>
+        <v>27.247104</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PC-1220</t>
+          <t>E1-2530</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>18.3</v>
+        <v>9</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>10.6872</v>
+        <v>5.255999999999999</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>92.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>92.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>9.832223999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PM-1006-SS</t>
+          <t>E2-0166</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>3.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>46.65</v>
+        <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>27.2436</v>
+        <v>0</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>97.00 pcs</t>
+          <t>0.00 pcs</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>97.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>26.426292</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>UA-1212</t>
+          <t>E2-0177</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>48.6</v>
+        <v>76.95</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>28.3824</v>
+        <v>44.9388</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>96.00 pcs</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -1576,13 +1612,13 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>27.247104</v>
+        <v>43.141248</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>E1-2530</t>
+          <t>E2-0545</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1591,29 +1627,29 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>9</v>
+        <v>147</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>5.255999999999999</v>
+        <v>85.848</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>96.00%</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0</v>
+        <v>82.41408</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>E2-0166</t>
+          <t>E2-0154</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1644,7 +1680,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>E2-0177</t>
+          <t>E2-0611</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1653,10 +1689,10 @@
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>76.95</v>
+        <v>95.25</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>44.9388</v>
+        <v>55.626</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1669,49 +1705,49 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>43.141248</v>
+        <v>53.40096</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>E2-0545</t>
+          <t>BE9-2513 (Clear)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>16.83 ft</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>147</v>
+        <v>419</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>85.848</v>
+        <v>244.696</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>7.17 ft</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>96.00%</t>
+          <t>29.86%</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>82.41408</v>
+        <v>73.06894444444443</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>E2-0154</t>
+          <t>E9-2512 (Clear)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -1722,7 +1758,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -1737,131 +1773,131 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>E2-0611</t>
+          <t>BE9-2511 (Clear)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>95.25</v>
+        <v>0</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>55.626</v>
+        <v>0</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>96.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>53.40096</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BE9-2513 (Clear)</t>
+          <t>BE9-2515 (Clear)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>16.83 ft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>419</v>
+        <v>527</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>244.696</v>
+        <v>307.768</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>7.17 ft</t>
+          <t>21.00 ft</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>29.86%</t>
+          <t>87.50%</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>73.06894444444443</v>
+        <v>269.297</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>E9-2512 (Clear)</t>
+          <t>BE9-2514 (Clear)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>0</v>
+        <v>444</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0</v>
+        <v>259.296</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>21.00 ft</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>87.50%</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0</v>
+        <v>226.884</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BE9-2511 (Clear)</t>
+          <t>BE9-2578 (Clear)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>3.00 ft</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0</v>
+        <v>154.176</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>21.00 ft</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>87.50%</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0</v>
+        <v>134.904</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BE9-2515 (Clear)</t>
+          <t>E9-2519 (Clear)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1870,10 +1906,10 @@
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>527</v>
+        <v>85.05</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>307.768</v>
+        <v>49.6692</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1886,266 +1922,144 @@
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>269.297</v>
+        <v>43.46054999999999</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BE9-2514 (Clear)</t>
+          <t>Glass Area (Adjusted)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>3.00 ft</t>
+          <t>17.56 sqft</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>444</v>
+        <v>0</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>259.296</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>21.00 ft</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>87.50%</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="n">
-        <v>226.884</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BE9-2578 (Clear)</t>
+          <t>Door Area (to subtract from glass)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>3.00 ft</t>
+          <t>0.00 sqft</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>154.176</v>
+        <v>0</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>21.00 ft</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>87.50%</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="n">
-        <v>134.904</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>E9-2519 (Clear)</t>
+          <t>Joints Fabrication Labor</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>3.00 ft</t>
+          <t>4.00 joints</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>85.05</v>
+        <v>0</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>49.6692</v>
+        <v>0</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>21.00 ft</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>87.50%</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="n">
-        <v>43.46054999999999</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Glass Area (Adjusted)</t>
+          <t>Gasket (E2-0052)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>11.78 sqft</t>
+          <t>39.67 ft</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>0</v>
+        <v>405</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0</v>
+        <v>236.52</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr"/>
+          <t>460.33 ft</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>92.07%</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>217.75608</v>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Door Area (to subtract from glass)</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>21.00 sqft</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr"/>
+      <c r="F68" s="1" t="inlineStr">
+        <is>
+          <t>REUSABLE GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>1308.607522444444</v>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Joints Fabrication Labor</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>4.00 joints</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Gasket (E2-0052)</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>39.67 ft</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="n">
-        <v>405</v>
-      </c>
-      <c r="D70" s="2" t="n">
-        <v>236.52</v>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>460.33 ft</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>92.07%</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="n">
-        <v>217.75608</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Door (3' X 7')</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="F72" s="1" t="inlineStr">
-        <is>
-          <t>REUSABLE GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="n">
-        <v>1308.607522444444</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="F73" s="1" t="inlineStr">
+      <c r="F69" s="1" t="inlineStr">
         <is>
           <t>REUSABLE % OF DISCOUNTED GRAND TOTAL</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>80.91%</t>
         </is>

</xml_diff>

<commit_message>
Changed names for headers
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="11" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="111" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Residual Waste" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,7 +33,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -54,12 +52,6 @@
         <bgColor rgb="0090EE90"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -73,14 +65,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -457,7 +448,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1310,7 +1301,7 @@
     <row r="37">
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>ORIGINAL SYSTEM TOTAL</t>
+          <t>ORIGINAL ELEVATION TOTAL</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1344,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2206,7 +2197,7 @@
     <row r="37">
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>ORIGINAL SYSTEM TOTAL</t>
+          <t>ORIGINAL ELEVATION TOTAL</t>
         </is>
       </c>
     </row>
@@ -2238,966 +2229,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
-    <col width="2" customWidth="1" min="3" max="3"/>
-    <col width="2" customWidth="1" min="4" max="4"/>
-    <col width="76" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>System Input</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>YES 45TU FRONT SET(OG)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>PROFILES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Finish</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Clear</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Discounted Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Elevation Type</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Sill/Jamb Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>BE9-2513</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>16.00 ft</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>419</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>244.696</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Total Count</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Sill/Jamb Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>BE9-2513</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>12.00 ft</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>419</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>244.696</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Bays Wide</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Flush Filler</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>E9-2512</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>24.00 ft</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>150</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>87.59999999999999</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Bays Tall</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Two Piece Mullion Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>BE9-2511</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>24.00 ft</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>497</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>290.248</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Opening Width</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>144</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Horizontal Screw Spline Assembly</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>BE9-2515</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>12.00 ft</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>527</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>307.768</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Opening Height</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>96</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Head</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>BE9-2514</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>12.00 ft</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>444</v>
-      </c>
-      <c r="I8" s="3" t="n">
-        <v>259.296</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Sq Ft per Type</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>96</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Thermal Sill Flashing</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>BE9-2578</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>12.00 ft</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>264</v>
-      </c>
-      <c r="I9" s="3" t="n">
-        <v>154.176</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Total Sq Ft</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>96</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Glass Stop (Use with BE9-2514, BE9-2515, BE9-2517)</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>E9-2519</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>24.00 ft</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="n">
-        <v>85.05</v>
-      </c>
-      <c r="I10" s="3" t="n">
-        <v>49.6692</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Perimeter Ft</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Total Perimeter Ft</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>40</v>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>ACCESSORIES</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>Doors</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1 x Narrow Door ($1,943.25)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Discounted Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>End Dam For Sill Flashing</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>E1-0199</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2.00 pcs</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Water Deflector</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>E2-0047</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>8.00 pcs</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>#12 x 1-1/4” PHSMS Type AB, Zinc Plated Steel, For Screw Spline Attachment</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>PC-1220</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>56.00 pcs</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>#10-24 x 3/8” PHMS, Stainless Steel, For Attachment of Sill to Sill Flashing</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>PM-1006-SS</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>12.00 pcs</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>#12 x 3/4” UFHSMS Type A, Zinc Plated Steel For End Dam Attachment</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>UA-1212</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>4.00 pcs</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Setting Block Chair Use with E2-0177 Setting Block at Sill</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>E1-2530</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>8.00 pcs</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="n">
-        <v>36</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>21.024</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Side Block For Intermediate Vertical Shallow Pocket</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>E2-0166</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>6.00 pcs</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Setting Block For Sill</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>E2-0177</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>8.00 pcs</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>1-1/8” “W” Side Block For Jamb</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>E2-0545</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>4.00 pcs</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>1/2” “W” Side Block For Intermediate Vertical Deep Pocket</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>E2-0154</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>6.00 pcs</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Setting Block For Intermediate Horizontal</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>E2-0611</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>8.00 pcs</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="E25" s="1" t="inlineStr">
-        <is>
-          <t>GLASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>Discounted Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Glass Area (Adjusted)</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>50.16 sqft</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="n">
-        <v>526.6799999999999</v>
-      </c>
-      <c r="I27" s="3" t="n">
-        <v>526.6799999999999</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="E28" s="1" t="inlineStr">
-        <is>
-          <t>DOORS</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>Discounted Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Door Area (to subtract from glass)</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>54.00 sqft</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="E31" s="1" t="inlineStr">
-        <is>
-          <t>FABRICATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Discounted Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Joints Fabrication Labor</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>24.00 joints</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="n">
-        <v>360</v>
-      </c>
-      <c r="I33" s="3" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="E34" s="1" t="inlineStr">
-        <is>
-          <t>GLAZING GASKET</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>Discounted Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Gasket</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>E2-0052</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>224.00 ft</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="n">
-        <v>405</v>
-      </c>
-      <c r="I36" s="3" t="n">
-        <v>236.52</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="E37" s="1" t="inlineStr">
-        <is>
-          <t>DOOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>Discounted Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Door (6' X 9')</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="n">
-        <v>1943.25</v>
-      </c>
-      <c r="I39" s="3" t="n">
-        <v>1943.25</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>ORIGINAL SYSTEM TOTAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="I41" s="3" t="n">
-        <v>6075.98</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>DISCOUNTED SYSTEM TOTAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="I43" s="3" t="n">
-        <v>4725.6232</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
@@ -3206,7 +2244,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Part Number / Description</t>
+          <t>Project Total Materials</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -3216,27 +2254,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Original Total Price</t>
+          <t>Original Total List Price</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Discounted Total Price</t>
+          <t>Discounted Total List Price</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Reusable Material Quantity</t>
+          <t>Residual Material Quantity</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Reusable % of Total</t>
+          <t>Residual Waste %</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Reusable Material Cost</t>
+          <t>Residual Material Cost</t>
         </is>
       </c>
     </row>
@@ -3248,7 +2286,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -3259,16 +2297,16 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>14.00 pcs</t>
+          <t>16.00 pcs</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>42.86%</t>
+          <t>25.00%</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
-        <v>26.49024</v>
+        <v>30.27456</v>
       </c>
     </row>
     <row r="3">
@@ -3279,7 +2317,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>24.00 pcs</t>
+          <t>16.00 pcs</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
@@ -3290,16 +2328,16 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>26.00 pcs</t>
+          <t>34.00 pcs</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>92.31%</t>
+          <t>47.06%</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
-        <v>36.13791999999999</v>
+        <v>47.25728</v>
       </c>
     </row>
     <row r="4">
@@ -3310,7 +2348,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>168.00 pcs</t>
+          <t>112.00 pcs</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
@@ -3321,7 +2359,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>32.00 pcs</t>
+          <t>88.00 pcs</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -3330,7 +2368,7 @@
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>3.419904</v>
+        <v>9.404736</v>
       </c>
     </row>
     <row r="5">
@@ -3341,7 +2379,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>36.00 pcs</t>
+          <t>24.00 pcs</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -3352,16 +2390,16 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>64.00 pcs</t>
+          <t>76.00 pcs</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>56.25%</t>
+          <t>31.58%</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
-        <v>17.435904</v>
+        <v>20.705136</v>
       </c>
     </row>
     <row r="6">
@@ -3372,7 +2410,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -3383,16 +2421,16 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>88.00 pcs</t>
+          <t>92.00 pcs</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>13.64%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>24.976512</v>
+        <v>26.111808</v>
       </c>
     </row>
     <row r="7">
@@ -3403,14 +2441,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>24.00 pcs</t>
+          <t>16.00 pcs</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>63.072</v>
+        <v>42.04799999999999</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -3434,7 +2472,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>18.00 pcs</t>
+          <t>12.00 pcs</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
@@ -3445,16 +2483,16 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>32.00 pcs</t>
+          <t>38.00 pcs</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>56.25%</t>
+          <t>31.58%</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">
-        <v>28.760832</v>
+        <v>34.153488</v>
       </c>
     </row>
     <row r="9">
@@ -3465,7 +2503,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>24.00 pcs</t>
+          <t>16.00 pcs</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -3476,16 +2514,16 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>26.00 pcs</t>
+          <t>34.00 pcs</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>92.31%</t>
+          <t>47.06%</t>
         </is>
       </c>
       <c r="G9" s="3" t="n">
-        <v>23.368176</v>
+        <v>30.558384</v>
       </c>
     </row>
     <row r="10">
@@ -3496,7 +2534,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
@@ -3507,16 +2545,16 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>38.00 pcs</t>
+          <t>42.00 pcs</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>31.58%</t>
+          <t>19.05%</t>
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>65.24448</v>
+        <v>72.11232</v>
       </c>
     </row>
     <row r="11">
@@ -3527,7 +2565,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.00 pcs</t>
+          <t>12.00 pcs</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -3538,16 +2576,16 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>32.00 pcs</t>
+          <t>38.00 pcs</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>56.25%</t>
+          <t>31.58%</t>
         </is>
       </c>
       <c r="G11" s="3" t="n">
-        <v>21.192192</v>
+        <v>25.165728</v>
       </c>
     </row>
     <row r="12">
@@ -3558,7 +2596,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>24.00 pcs</t>
+          <t>16.00 pcs</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
@@ -3569,16 +2607,16 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>26.00 pcs</t>
+          <t>34.00 pcs</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>92.31%</t>
+          <t>47.06%</t>
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.92552</v>
+        <v>37.82568</v>
       </c>
     </row>
     <row r="13">
@@ -3589,18 +2627,18 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>84.00 ft</t>
+          <t>56.00 ft</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1676</v>
+        <v>1257</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>978.784</v>
+        <v>734.088</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>8.00 x3, 12.00 ft</t>
+          <t>8.00 x2 ft</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -3609,7 +2647,7 @@
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>367.044</v>
+        <v>163.1306666666667</v>
       </c>
     </row>
     <row r="14">
@@ -3620,14 +2658,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>72.00 ft</t>
+          <t>48.00 ft</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>262.8</v>
+        <v>175.2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -3651,14 +2689,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>72.00 ft</t>
+          <t>48.00 ft</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1491</v>
+        <v>994</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>870.7439999999999</v>
+        <v>580.496</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -3682,27 +2720,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>36.00 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>1054</v>
+        <v>527</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>615.5359999999999</v>
+        <v>307.768</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>153.884</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -3713,27 +2751,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>36.00 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>888</v>
+        <v>444</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>518.592</v>
+        <v>259.296</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G17" s="3" t="n">
-        <v>129.648</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3744,27 +2782,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>36.00 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>528</v>
+        <v>264</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>308.352</v>
+        <v>154.176</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>12.00 ft</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G18" s="3" t="n">
-        <v>77.08799999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -3775,14 +2813,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>72.00 ft</t>
+          <t>48.00 ft</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>255.15</v>
+        <v>170.1</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>149.0076</v>
+        <v>99.33839999999999</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3806,7 +2844,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>217.66 sqft</t>
+          <t>167.50 sqft</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -3835,7 +2873,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>54.00 sqft</t>
+          <t>0.00 sqft</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -3864,7 +2902,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>72.00 joints</t>
+          <t>48.00 joints</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -3893,18 +2931,18 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>672.00 ft</t>
+          <t>448.00 ft</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>810</v>
+        <v>405</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>473.04</v>
+        <v>236.52</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>52.00, 276.00 ft</t>
+          <t>52.00 ft</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3913,479 +2951,28 @@
         </is>
       </c>
       <c r="G23" s="3" t="n">
-        <v>155.15712</v>
+        <v>24.59808</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Door (6' X 9')</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>1.00 pcs</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>REUSABLE GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>521.2978666666667</v>
+      </c>
     </row>
     <row r="25">
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>REUSABLE GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="n">
-        <v>1158.7728</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="F26" s="5" t="inlineStr">
-        <is>
           <t>REUSABLE % OF RUNNING GRAND TOTAL</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>24.71%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Finish</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>Leftover Quantity</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>BE9-2513-clear</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>clear</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>36</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>E9-2512-clear</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>clear</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BE9-2511-clear</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>clear</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BE9-2515-clear</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>clear</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>12</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>BE9-2514-clear</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>clear</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>BE9-2578-clear</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>clear</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>12</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>E9-2519-clear</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>clear</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>E1-0199</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>14</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>E2-0047</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>26</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>PC-1220</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>32</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>PM-1006-SS</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>64</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>UA-1212</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>88</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>E1-2530</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>E2-0166</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>32</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>E2-0177</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>26</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>E2-0545</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>38</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>E2-0154</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>32</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>E2-0611</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>26</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>E2-0052</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>328</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>ft</t>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>17.16%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Glazing Gasket not manual
</commit_message>
<xml_diff>
--- a/projects/1_Report.xlsx
+++ b/projects/1_Report.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="2" customWidth="1" min="4" max="4"/>
     <col width="76" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="28" customWidth="1" min="9" max="9"/>
   </cols>
@@ -530,7 +530,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.67 ft x 10</t>
+          <t>0.17 ft</t>
         </is>
       </c>
       <c r="H3" s="3" t="n">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -561,14 +561,14 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.83 ft x 10</t>
+          <t>0.08 ft</t>
         </is>
       </c>
       <c r="H4" s="3" t="n">
-        <v>419</v>
+        <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>244.696</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -592,7 +592,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.00 ft x 10</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="H5" s="3" t="n">
@@ -623,7 +623,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.00 ft x 10</t>
+          <t>0.00 ft</t>
         </is>
       </c>
       <c r="H6" s="3" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.00 ft</t>
+          <t>1.00 ft</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.83 ft x 10</t>
+          <t>0.08 ft</t>
         </is>
       </c>
       <c r="H7" s="3" t="n">
@@ -674,7 +674,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10.00 ft</t>
+          <t>1.00 ft</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.83 ft x 10</t>
+          <t>0.08 ft</t>
         </is>
       </c>
       <c r="H8" s="3" t="n">
@@ -707,7 +707,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0.69 sqft</t>
+          <t>0.01 sqft</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.83 ft x 10</t>
+          <t>0.08 ft</t>
         </is>
       </c>
       <c r="H9" s="3" t="n">
@@ -740,7 +740,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>6.94 sqft</t>
+          <t>0.01 sqft</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.83 ft x 10</t>
+          <t>0.08 ft</t>
         </is>
       </c>
       <c r="H10" s="3" t="n">
@@ -773,7 +773,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3.33 ft</t>
+          <t>0.33 ft</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>33.33 ft</t>
+          <t>0.33 ft</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H14" s="3" t="n">
@@ -867,7 +867,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H15" s="3" t="n">
@@ -890,7 +890,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>80.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="H16" s="3" t="n">
@@ -913,7 +913,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>30.00 pcs</t>
+          <t>3.00 pcs</t>
         </is>
       </c>
       <c r="H17" s="3" t="n">
@@ -936,7 +936,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>40.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="H18" s="3" t="n">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H21" s="3" t="n">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H22" s="3" t="n">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="H24" s="3" t="n">
@@ -1085,255 +1085,221 @@
       </c>
     </row>
     <row r="25">
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Glazing Gasket For 1” Glazing</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>E2-0052</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0.67 pcs</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>0.47304</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>GLASS</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="E26" s="2" t="inlineStr">
+    <row r="27">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Part Number</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Original Price</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Discounted Price</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="E27" t="inlineStr">
+    <row r="28">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Glass Area (Adjusted)</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2.50 sqft</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="n">
-        <v>26.25</v>
-      </c>
-      <c r="I27" s="3" t="n">
-        <v>26.25</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="E28" s="1" t="inlineStr">
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0.06 sqft</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>0.65625</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>0.65625</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>DOORS</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="E29" s="2" t="inlineStr">
+    <row r="30">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Part Number</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Original Price</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Discounted Price</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="E30" t="inlineStr">
+    <row r="31">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Door Area (to subtract from glass)</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>0.00 sqft</t>
         </is>
       </c>
-      <c r="H30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="E31" s="1" t="inlineStr">
+      <c r="H31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>FABRICATION</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="E32" s="2" t="inlineStr">
+    <row r="33">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Part Number</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Original Price</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>Discounted Price</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="E33" t="inlineStr">
+    <row r="34">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Joints Fabrication Labor</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>40.00 joints</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="n">
-        <v>600</v>
-      </c>
-      <c r="I33" s="3" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="E34" s="1" t="inlineStr">
-        <is>
-          <t>GLAZING GASKET</t>
-        </is>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>4.00 joints</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="35">
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Part Number</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Original Price</t>
-        </is>
-      </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Discounted Price</t>
+          <t>ORIGINAL ELEVATION TOTAL</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Gasket</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>E2-0052</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>66.67 pcs</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="n">
-        <v>405</v>
-      </c>
       <c r="I36" s="3" t="n">
-        <v>236.52</v>
+        <v>2426.06625</v>
       </c>
     </row>
     <row r="37">
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>ORIGINAL ELEVATION TOTAL</t>
+          <t>DISCOUNTED ELEVATION TOTAL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="I38" s="3" t="n">
-        <v>3814.85</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>DISCOUNTED ELEVATION TOTAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="I40" s="3" t="n">
-        <v>2488.3924</v>
+        <v>1442.05569</v>
       </c>
     </row>
   </sheetData>
@@ -1351,7 +1317,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -1404,7 +1370,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -1415,16 +1381,16 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>18.00 pcs</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>11.11%</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0</v>
+        <v>34.05887999999999</v>
       </c>
     </row>
     <row r="3">
@@ -1435,7 +1401,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
@@ -1446,16 +1412,16 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>30.00 pcs</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>4.17%</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
-        <v>41.69759999999999</v>
+        <v>66.71615999999999</v>
       </c>
     </row>
     <row r="4">
@@ -1466,7 +1432,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>80.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
@@ -1477,16 +1443,16 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>92.00 pcs</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2.13744</v>
+        <v>9.832223999999998</v>
       </c>
     </row>
     <row r="5">
@@ -1497,7 +1463,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30.00 pcs</t>
+          <t>3.00 pcs</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -1508,16 +1474,16 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>70.00 pcs</t>
+          <t>97.00 pcs</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>42.86%</t>
+          <t>3.09%</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
-        <v>19.07052</v>
+        <v>26.426292</v>
       </c>
     </row>
     <row r="6">
@@ -1528,7 +1494,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>40.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -1539,16 +1505,16 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>60.00 pcs</t>
+          <t>96.00 pcs</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>4.17%</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>17.02944</v>
+        <v>27.247104</v>
       </c>
     </row>
     <row r="7">
@@ -1621,7 +1587,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -1632,16 +1598,16 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>30.00 pcs</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>4.17%</t>
         </is>
       </c>
       <c r="G9" s="3" t="n">
-        <v>26.96328</v>
+        <v>43.141248</v>
       </c>
     </row>
     <row r="10">
@@ -1652,7 +1618,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
@@ -1663,16 +1629,16 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>30.00 pcs</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>4.17%</t>
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>51.5088</v>
+        <v>82.41408</v>
       </c>
     </row>
     <row r="11">
@@ -1714,7 +1680,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>20.00 pcs</t>
+          <t>2.00 pcs</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
@@ -1725,16 +1691,16 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>30.00 pcs</t>
+          <t>48.00 pcs</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>4.17%</t>
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>33.3756</v>
+        <v>53.40096</v>
       </c>
     </row>
     <row r="13">
@@ -1745,27 +1711,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>25.00 ft</t>
+          <t>0.25 ft</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>838</v>
+        <v>419</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>489.392</v>
+        <v>244.696</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.67 ft, 22.33 ft</t>
+          <t>23.75 ft</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>1.05%</t>
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>234.5003333333333</v>
+        <v>242.1470833333333</v>
       </c>
     </row>
     <row r="14">
@@ -1838,7 +1804,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>8.33 ft</t>
+          <t>0.08 ft</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -1849,16 +1815,16 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>15.67 ft</t>
+          <t>23.92 ft</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>53.19%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>200.9041111111112</v>
+        <v>306.6993611111111</v>
       </c>
     </row>
     <row r="17">
@@ -1869,7 +1835,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>8.33 ft</t>
+          <t>0.08 ft</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
@@ -1880,16 +1846,16 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>15.67 ft</t>
+          <t>23.92 ft</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>53.19%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="G17" s="3" t="n">
-        <v>169.2626666666668</v>
+        <v>258.3956666666667</v>
       </c>
     </row>
     <row r="18">
@@ -1900,7 +1866,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.33 ft</t>
+          <t>0.08 ft</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -1911,16 +1877,16 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>15.67 ft</t>
+          <t>23.92 ft</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>53.19%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="G18" s="3" t="n">
-        <v>100.6426666666667</v>
+        <v>153.6406666666667</v>
       </c>
     </row>
     <row r="19">
@@ -1931,7 +1897,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8.33 ft</t>
+          <t>0.08 ft</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -1942,56 +1908,58 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>15.67 ft</t>
+          <t>23.92 ft</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>53.19%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="G19" s="3" t="n">
-        <v>32.42295000000001</v>
+        <v>49.4967375</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Glass Area (Adjusted)</t>
+          <t>E2-0052</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2.50 sqft</t>
+          <t>0.67 pcs</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0</v>
+        <v>0.47304</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
+          <t>0.33 pcs</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.157664232</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Door Area (to subtract from glass)</t>
+          <t>Glass Area (Adjusted)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0.00 sqft</t>
+          <t>0.06 sqft</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -2015,12 +1983,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Joints Fabrication Labor</t>
+          <t>Door Area (to subtract from glass)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>40.00 joints</t>
+          <t>0.00 sqft</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -2044,33 +2012,31 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gasket (E2-0052)</t>
+          <t>Joints Fabrication Labor</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>66.67 pcs</t>
+          <t>4.00 joints</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>405</v>
+        <v>0</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>236.52</v>
+        <v>0</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>433.33 pcs</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>15.38%</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>204.984</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="F24" s="6" t="inlineStr">
@@ -2079,7 +2045,7 @@
         </is>
       </c>
       <c r="G24" s="3" t="n">
-        <v>1134.499407777778</v>
+        <v>1353.774127509778</v>
       </c>
     </row>
     <row r="25">
@@ -2090,7 +2056,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>60.92%</t>
+          <t>98.00%</t>
         </is>
       </c>
     </row>

</xml_diff>